<commit_message>
Updating the models for Rosiori and MM&MV
</commit_message>
<xml_diff>
--- a/Market Fundamentals/Transelectrica_data/Cons_Prod_final/Weekly_Consumption_2026.xlsx
+++ b/Market Fundamentals/Transelectrica_data/Cons_Prod_final/Weekly_Consumption_2026.xlsx
@@ -44272,7 +44272,7 @@
         <v>1</v>
       </c>
       <c r="C2498">
-        <v>5880</v>
+        <v>5700</v>
       </c>
       <c r="D2498" t="s">
         <v>2500</v>
@@ -44286,7 +44286,7 @@
         <v>2</v>
       </c>
       <c r="C2499">
-        <v>5820</v>
+        <v>5650</v>
       </c>
       <c r="D2499" t="s">
         <v>2501</v>
@@ -44300,7 +44300,7 @@
         <v>3</v>
       </c>
       <c r="C2500">
-        <v>5770</v>
+        <v>5590</v>
       </c>
       <c r="D2500" t="s">
         <v>2502</v>
@@ -44314,7 +44314,7 @@
         <v>4</v>
       </c>
       <c r="C2501">
-        <v>5720</v>
+        <v>5540</v>
       </c>
       <c r="D2501" t="s">
         <v>2503</v>
@@ -44328,7 +44328,7 @@
         <v>5</v>
       </c>
       <c r="C2502">
-        <v>5660</v>
+        <v>5500</v>
       </c>
       <c r="D2502" t="s">
         <v>2504</v>
@@ -44342,7 +44342,7 @@
         <v>6</v>
       </c>
       <c r="C2503">
-        <v>5620</v>
+        <v>5460</v>
       </c>
       <c r="D2503" t="s">
         <v>2505</v>
@@ -44356,7 +44356,7 @@
         <v>7</v>
       </c>
       <c r="C2504">
-        <v>5600</v>
+        <v>5430</v>
       </c>
       <c r="D2504" t="s">
         <v>2506</v>
@@ -44370,7 +44370,7 @@
         <v>8</v>
       </c>
       <c r="C2505">
-        <v>5570</v>
+        <v>5410</v>
       </c>
       <c r="D2505" t="s">
         <v>2507</v>
@@ -44384,7 +44384,7 @@
         <v>9</v>
       </c>
       <c r="C2506">
-        <v>5550</v>
+        <v>5400</v>
       </c>
       <c r="D2506" t="s">
         <v>2508</v>
@@ -44398,7 +44398,7 @@
         <v>10</v>
       </c>
       <c r="C2507">
-        <v>5530</v>
+        <v>5400</v>
       </c>
       <c r="D2507" t="s">
         <v>2509</v>
@@ -44412,7 +44412,7 @@
         <v>11</v>
       </c>
       <c r="C2508">
-        <v>5510</v>
+        <v>5380</v>
       </c>
       <c r="D2508" t="s">
         <v>2510</v>
@@ -44426,7 +44426,7 @@
         <v>12</v>
       </c>
       <c r="C2509">
-        <v>5490</v>
+        <v>5380</v>
       </c>
       <c r="D2509" t="s">
         <v>2511</v>
@@ -44440,7 +44440,7 @@
         <v>13</v>
       </c>
       <c r="C2510">
-        <v>5480</v>
+        <v>5370</v>
       </c>
       <c r="D2510" t="s">
         <v>2512</v>
@@ -44454,7 +44454,7 @@
         <v>14</v>
       </c>
       <c r="C2511">
-        <v>5460</v>
+        <v>5370</v>
       </c>
       <c r="D2511" t="s">
         <v>2513</v>
@@ -44468,7 +44468,7 @@
         <v>15</v>
       </c>
       <c r="C2512">
-        <v>5450</v>
+        <v>5380</v>
       </c>
       <c r="D2512" t="s">
         <v>2514</v>
@@ -44482,7 +44482,7 @@
         <v>16</v>
       </c>
       <c r="C2513">
-        <v>5450</v>
+        <v>5390</v>
       </c>
       <c r="D2513" t="s">
         <v>2515</v>
@@ -44496,7 +44496,7 @@
         <v>17</v>
       </c>
       <c r="C2514">
-        <v>5460</v>
+        <v>5400</v>
       </c>
       <c r="D2514" t="s">
         <v>2516</v>
@@ -44510,7 +44510,7 @@
         <v>18</v>
       </c>
       <c r="C2515">
-        <v>5480</v>
+        <v>5420</v>
       </c>
       <c r="D2515" t="s">
         <v>2517</v>
@@ -44524,7 +44524,7 @@
         <v>19</v>
       </c>
       <c r="C2516">
-        <v>5500</v>
+        <v>5440</v>
       </c>
       <c r="D2516" t="s">
         <v>2518</v>
@@ -44538,7 +44538,7 @@
         <v>20</v>
       </c>
       <c r="C2517">
-        <v>5540</v>
+        <v>5480</v>
       </c>
       <c r="D2517" t="s">
         <v>2519</v>
@@ -44552,7 +44552,7 @@
         <v>21</v>
       </c>
       <c r="C2518">
-        <v>5590</v>
+        <v>5540</v>
       </c>
       <c r="D2518" t="s">
         <v>2520</v>
@@ -44566,7 +44566,7 @@
         <v>22</v>
       </c>
       <c r="C2519">
-        <v>5650</v>
+        <v>5620</v>
       </c>
       <c r="D2519" t="s">
         <v>2521</v>
@@ -44580,7 +44580,7 @@
         <v>23</v>
       </c>
       <c r="C2520">
-        <v>5730</v>
+        <v>5720</v>
       </c>
       <c r="D2520" t="s">
         <v>2522</v>
@@ -44608,7 +44608,7 @@
         <v>25</v>
       </c>
       <c r="C2522">
-        <v>5940</v>
+        <v>5970</v>
       </c>
       <c r="D2522" t="s">
         <v>2524</v>
@@ -44622,7 +44622,7 @@
         <v>26</v>
       </c>
       <c r="C2523">
-        <v>6070</v>
+        <v>6100</v>
       </c>
       <c r="D2523" t="s">
         <v>2525</v>
@@ -44636,7 +44636,7 @@
         <v>27</v>
       </c>
       <c r="C2524">
-        <v>6210</v>
+        <v>6230</v>
       </c>
       <c r="D2524" t="s">
         <v>2526</v>
@@ -44650,7 +44650,7 @@
         <v>28</v>
       </c>
       <c r="C2525">
-        <v>6350</v>
+        <v>6360</v>
       </c>
       <c r="D2525" t="s">
         <v>2527</v>
@@ -44664,7 +44664,7 @@
         <v>29</v>
       </c>
       <c r="C2526">
-        <v>6500</v>
+        <v>6470</v>
       </c>
       <c r="D2526" t="s">
         <v>2528</v>
@@ -44678,7 +44678,7 @@
         <v>30</v>
       </c>
       <c r="C2527">
-        <v>6630</v>
+        <v>6570</v>
       </c>
       <c r="D2527" t="s">
         <v>2529</v>
@@ -44692,7 +44692,7 @@
         <v>31</v>
       </c>
       <c r="C2528">
-        <v>6750</v>
+        <v>6660</v>
       </c>
       <c r="D2528" t="s">
         <v>2530</v>
@@ -44706,7 +44706,7 @@
         <v>32</v>
       </c>
       <c r="C2529">
-        <v>6850</v>
+        <v>6720</v>
       </c>
       <c r="D2529" t="s">
         <v>2531</v>
@@ -44720,7 +44720,7 @@
         <v>33</v>
       </c>
       <c r="C2530">
-        <v>6950</v>
+        <v>6760</v>
       </c>
       <c r="D2530" t="s">
         <v>2532</v>
@@ -44734,7 +44734,7 @@
         <v>34</v>
       </c>
       <c r="C2531">
-        <v>7000</v>
+        <v>6770</v>
       </c>
       <c r="D2531" t="s">
         <v>2533</v>
@@ -44748,7 +44748,7 @@
         <v>35</v>
       </c>
       <c r="C2532">
-        <v>7000</v>
+        <v>6760</v>
       </c>
       <c r="D2532" t="s">
         <v>2534</v>
@@ -44762,7 +44762,7 @@
         <v>36</v>
       </c>
       <c r="C2533">
-        <v>6970</v>
+        <v>6740</v>
       </c>
       <c r="D2533" t="s">
         <v>2535</v>
@@ -44776,7 +44776,7 @@
         <v>37</v>
       </c>
       <c r="C2534">
-        <v>6900</v>
+        <v>6680</v>
       </c>
       <c r="D2534" t="s">
         <v>2536</v>
@@ -44790,7 +44790,7 @@
         <v>38</v>
       </c>
       <c r="C2535">
-        <v>6820</v>
+        <v>6630</v>
       </c>
       <c r="D2535" t="s">
         <v>2537</v>
@@ -44804,7 +44804,7 @@
         <v>39</v>
       </c>
       <c r="C2536">
-        <v>6730</v>
+        <v>6560</v>
       </c>
       <c r="D2536" t="s">
         <v>2538</v>
@@ -44818,7 +44818,7 @@
         <v>40</v>
       </c>
       <c r="C2537">
-        <v>6630</v>
+        <v>6480</v>
       </c>
       <c r="D2537" t="s">
         <v>2539</v>
@@ -44832,7 +44832,7 @@
         <v>41</v>
       </c>
       <c r="C2538">
-        <v>6530</v>
+        <v>6400</v>
       </c>
       <c r="D2538" t="s">
         <v>2540</v>
@@ -44846,7 +44846,7 @@
         <v>42</v>
       </c>
       <c r="C2539">
-        <v>6430</v>
+        <v>6320</v>
       </c>
       <c r="D2539" t="s">
         <v>2541</v>
@@ -44860,7 +44860,7 @@
         <v>43</v>
       </c>
       <c r="C2540">
-        <v>6340</v>
+        <v>6240</v>
       </c>
       <c r="D2540" t="s">
         <v>2542</v>
@@ -44874,7 +44874,7 @@
         <v>44</v>
       </c>
       <c r="C2541">
-        <v>6260</v>
+        <v>6170</v>
       </c>
       <c r="D2541" t="s">
         <v>2543</v>
@@ -44888,7 +44888,7 @@
         <v>45</v>
       </c>
       <c r="C2542">
-        <v>6190</v>
+        <v>6110</v>
       </c>
       <c r="D2542" t="s">
         <v>2544</v>
@@ -44902,7 +44902,7 @@
         <v>46</v>
       </c>
       <c r="C2543">
-        <v>6140</v>
+        <v>6050</v>
       </c>
       <c r="D2543" t="s">
         <v>2545</v>
@@ -44916,7 +44916,7 @@
         <v>47</v>
       </c>
       <c r="C2544">
-        <v>6100</v>
+        <v>6010</v>
       </c>
       <c r="D2544" t="s">
         <v>2546</v>
@@ -44930,7 +44930,7 @@
         <v>48</v>
       </c>
       <c r="C2545">
-        <v>6070</v>
+        <v>5980</v>
       </c>
       <c r="D2545" t="s">
         <v>2547</v>
@@ -44944,7 +44944,7 @@
         <v>49</v>
       </c>
       <c r="C2546">
-        <v>6060</v>
+        <v>5960</v>
       </c>
       <c r="D2546" t="s">
         <v>2548</v>
@@ -44958,7 +44958,7 @@
         <v>50</v>
       </c>
       <c r="C2547">
-        <v>6040</v>
+        <v>5950</v>
       </c>
       <c r="D2547" t="s">
         <v>2549</v>
@@ -44972,7 +44972,7 @@
         <v>51</v>
       </c>
       <c r="C2548">
-        <v>6030</v>
+        <v>5960</v>
       </c>
       <c r="D2548" t="s">
         <v>2550</v>
@@ -44986,7 +44986,7 @@
         <v>52</v>
       </c>
       <c r="C2549">
-        <v>6020</v>
+        <v>5970</v>
       </c>
       <c r="D2549" t="s">
         <v>2551</v>
@@ -45000,7 +45000,7 @@
         <v>53</v>
       </c>
       <c r="C2550">
-        <v>6030</v>
+        <v>5990</v>
       </c>
       <c r="D2550" t="s">
         <v>2552</v>
@@ -45014,7 +45014,7 @@
         <v>54</v>
       </c>
       <c r="C2551">
-        <v>6060</v>
+        <v>6020</v>
       </c>
       <c r="D2551" t="s">
         <v>2553</v>
@@ -45028,7 +45028,7 @@
         <v>55</v>
       </c>
       <c r="C2552">
-        <v>6130</v>
+        <v>6060</v>
       </c>
       <c r="D2552" t="s">
         <v>2554</v>
@@ -45042,7 +45042,7 @@
         <v>56</v>
       </c>
       <c r="C2553">
-        <v>6200</v>
+        <v>6100</v>
       </c>
       <c r="D2553" t="s">
         <v>2555</v>
@@ -45056,7 +45056,7 @@
         <v>57</v>
       </c>
       <c r="C2554">
-        <v>6260</v>
+        <v>6150</v>
       </c>
       <c r="D2554" t="s">
         <v>2556</v>
@@ -45070,7 +45070,7 @@
         <v>58</v>
       </c>
       <c r="C2555">
-        <v>6330</v>
+        <v>6200</v>
       </c>
       <c r="D2555" t="s">
         <v>2557</v>
@@ -45084,7 +45084,7 @@
         <v>59</v>
       </c>
       <c r="C2556">
-        <v>6380</v>
+        <v>6240</v>
       </c>
       <c r="D2556" t="s">
         <v>2558</v>
@@ -45098,7 +45098,7 @@
         <v>60</v>
       </c>
       <c r="C2557">
-        <v>6430</v>
+        <v>6290</v>
       </c>
       <c r="D2557" t="s">
         <v>2559</v>
@@ -45112,7 +45112,7 @@
         <v>61</v>
       </c>
       <c r="C2558">
-        <v>6480</v>
+        <v>6330</v>
       </c>
       <c r="D2558" t="s">
         <v>2560</v>
@@ -45126,7 +45126,7 @@
         <v>62</v>
       </c>
       <c r="C2559">
-        <v>6530</v>
+        <v>6380</v>
       </c>
       <c r="D2559" t="s">
         <v>2561</v>
@@ -45140,7 +45140,7 @@
         <v>63</v>
       </c>
       <c r="C2560">
-        <v>6570</v>
+        <v>6430</v>
       </c>
       <c r="D2560" t="s">
         <v>2562</v>
@@ -45154,7 +45154,7 @@
         <v>64</v>
       </c>
       <c r="C2561">
-        <v>6630</v>
+        <v>6490</v>
       </c>
       <c r="D2561" t="s">
         <v>2563</v>
@@ -45168,7 +45168,7 @@
         <v>65</v>
       </c>
       <c r="C2562">
-        <v>6690</v>
+        <v>6550</v>
       </c>
       <c r="D2562" t="s">
         <v>2564</v>
@@ -45182,7 +45182,7 @@
         <v>66</v>
       </c>
       <c r="C2563">
-        <v>6770</v>
+        <v>6630</v>
       </c>
       <c r="D2563" t="s">
         <v>2565</v>
@@ -45196,7 +45196,7 @@
         <v>67</v>
       </c>
       <c r="C2564">
-        <v>6850</v>
+        <v>6700</v>
       </c>
       <c r="D2564" t="s">
         <v>2566</v>
@@ -45210,7 +45210,7 @@
         <v>68</v>
       </c>
       <c r="C2565">
-        <v>6930</v>
+        <v>6790</v>
       </c>
       <c r="D2565" t="s">
         <v>2567</v>
@@ -45224,7 +45224,7 @@
         <v>69</v>
       </c>
       <c r="C2566">
-        <v>7020</v>
+        <v>6870</v>
       </c>
       <c r="D2566" t="s">
         <v>2568</v>
@@ -45238,7 +45238,7 @@
         <v>70</v>
       </c>
       <c r="C2567">
-        <v>7090</v>
+        <v>6960</v>
       </c>
       <c r="D2567" t="s">
         <v>2569</v>
@@ -45252,7 +45252,7 @@
         <v>71</v>
       </c>
       <c r="C2568">
-        <v>7160</v>
+        <v>7030</v>
       </c>
       <c r="D2568" t="s">
         <v>2570</v>
@@ -45266,7 +45266,7 @@
         <v>72</v>
       </c>
       <c r="C2569">
-        <v>7220</v>
+        <v>7100</v>
       </c>
       <c r="D2569" t="s">
         <v>2571</v>
@@ -45280,7 +45280,7 @@
         <v>73</v>
       </c>
       <c r="C2570">
-        <v>7310</v>
+        <v>7170</v>
       </c>
       <c r="D2570" t="s">
         <v>2572</v>
@@ -45294,7 +45294,7 @@
         <v>74</v>
       </c>
       <c r="C2571">
-        <v>7380</v>
+        <v>7240</v>
       </c>
       <c r="D2571" t="s">
         <v>2573</v>
@@ -45308,7 +45308,7 @@
         <v>75</v>
       </c>
       <c r="C2572">
-        <v>7440</v>
+        <v>7330</v>
       </c>
       <c r="D2572" t="s">
         <v>2574</v>
@@ -45322,7 +45322,7 @@
         <v>76</v>
       </c>
       <c r="C2573">
-        <v>7520</v>
+        <v>7420</v>
       </c>
       <c r="D2573" t="s">
         <v>2575</v>
@@ -45336,7 +45336,7 @@
         <v>77</v>
       </c>
       <c r="C2574">
-        <v>7610</v>
+        <v>7490</v>
       </c>
       <c r="D2574" t="s">
         <v>2576</v>
@@ -45350,7 +45350,7 @@
         <v>78</v>
       </c>
       <c r="C2575">
-        <v>7680</v>
+        <v>7570</v>
       </c>
       <c r="D2575" t="s">
         <v>2577</v>
@@ -45364,7 +45364,7 @@
         <v>79</v>
       </c>
       <c r="C2576">
-        <v>7700</v>
+        <v>7600</v>
       </c>
       <c r="D2576" t="s">
         <v>2578</v>
@@ -45378,7 +45378,7 @@
         <v>80</v>
       </c>
       <c r="C2577">
-        <v>7700</v>
+        <v>7630</v>
       </c>
       <c r="D2577" t="s">
         <v>2579</v>
@@ -45392,7 +45392,7 @@
         <v>81</v>
       </c>
       <c r="C2578">
-        <v>7680</v>
+        <v>7610</v>
       </c>
       <c r="D2578" t="s">
         <v>2580</v>
@@ -45406,7 +45406,7 @@
         <v>82</v>
       </c>
       <c r="C2579">
-        <v>7630</v>
+        <v>7580</v>
       </c>
       <c r="D2579" t="s">
         <v>2581</v>
@@ -45420,7 +45420,7 @@
         <v>83</v>
       </c>
       <c r="C2580">
-        <v>7570</v>
+        <v>7510</v>
       </c>
       <c r="D2580" t="s">
         <v>2582</v>
@@ -45434,7 +45434,7 @@
         <v>84</v>
       </c>
       <c r="C2581">
-        <v>7480</v>
+        <v>7420</v>
       </c>
       <c r="D2581" t="s">
         <v>2583</v>
@@ -45448,7 +45448,7 @@
         <v>85</v>
       </c>
       <c r="C2582">
-        <v>7370</v>
+        <v>7330</v>
       </c>
       <c r="D2582" t="s">
         <v>2584</v>
@@ -45462,7 +45462,7 @@
         <v>86</v>
       </c>
       <c r="C2583">
-        <v>7270</v>
+        <v>7220</v>
       </c>
       <c r="D2583" t="s">
         <v>2585</v>
@@ -45476,7 +45476,7 @@
         <v>87</v>
       </c>
       <c r="C2584">
-        <v>7180</v>
+        <v>7110</v>
       </c>
       <c r="D2584" t="s">
         <v>2586</v>
@@ -45490,7 +45490,7 @@
         <v>88</v>
       </c>
       <c r="C2585">
-        <v>7040</v>
+        <v>7000</v>
       </c>
       <c r="D2585" t="s">
         <v>2587</v>
@@ -45504,7 +45504,7 @@
         <v>89</v>
       </c>
       <c r="C2586">
-        <v>6890</v>
+        <v>6870</v>
       </c>
       <c r="D2586" t="s">
         <v>2588</v>
@@ -45518,7 +45518,7 @@
         <v>90</v>
       </c>
       <c r="C2587">
-        <v>6760</v>
+        <v>6730</v>
       </c>
       <c r="D2587" t="s">
         <v>2589</v>
@@ -45532,7 +45532,7 @@
         <v>91</v>
       </c>
       <c r="C2588">
-        <v>6600</v>
+        <v>6580</v>
       </c>
       <c r="D2588" t="s">
         <v>2590</v>
@@ -45546,7 +45546,7 @@
         <v>92</v>
       </c>
       <c r="C2589">
-        <v>6460</v>
+        <v>6420</v>
       </c>
       <c r="D2589" t="s">
         <v>2591</v>
@@ -45560,7 +45560,7 @@
         <v>93</v>
       </c>
       <c r="C2590">
-        <v>6300</v>
+        <v>6280</v>
       </c>
       <c r="D2590" t="s">
         <v>2592</v>
@@ -45574,7 +45574,7 @@
         <v>94</v>
       </c>
       <c r="C2591">
-        <v>6150</v>
+        <v>6140</v>
       </c>
       <c r="D2591" t="s">
         <v>2593</v>
@@ -45588,7 +45588,7 @@
         <v>95</v>
       </c>
       <c r="C2592">
-        <v>6030</v>
+        <v>6000</v>
       </c>
       <c r="D2592" t="s">
         <v>2594</v>
@@ -45616,7 +45616,7 @@
         <v>1</v>
       </c>
       <c r="C2594">
-        <v>5760</v>
+        <v>5880</v>
       </c>
       <c r="D2594" t="s">
         <v>2596</v>
@@ -45630,7 +45630,7 @@
         <v>2</v>
       </c>
       <c r="C2595">
-        <v>5680</v>
+        <v>5830</v>
       </c>
       <c r="D2595" t="s">
         <v>2597</v>
@@ -45644,7 +45644,7 @@
         <v>3</v>
       </c>
       <c r="C2596">
-        <v>5610</v>
+        <v>5770</v>
       </c>
       <c r="D2596" t="s">
         <v>2598</v>
@@ -45658,7 +45658,7 @@
         <v>4</v>
       </c>
       <c r="C2597">
-        <v>5560</v>
+        <v>5710</v>
       </c>
       <c r="D2597" t="s">
         <v>2599</v>
@@ -45672,7 +45672,7 @@
         <v>5</v>
       </c>
       <c r="C2598">
-        <v>5520</v>
+        <v>5650</v>
       </c>
       <c r="D2598" t="s">
         <v>2600</v>
@@ -45686,7 +45686,7 @@
         <v>6</v>
       </c>
       <c r="C2599">
-        <v>5490</v>
+        <v>5610</v>
       </c>
       <c r="D2599" t="s">
         <v>2601</v>
@@ -45700,7 +45700,7 @@
         <v>7</v>
       </c>
       <c r="C2600">
-        <v>5460</v>
+        <v>5570</v>
       </c>
       <c r="D2600" t="s">
         <v>2602</v>
@@ -45714,7 +45714,7 @@
         <v>8</v>
       </c>
       <c r="C2601">
-        <v>5430</v>
+        <v>5540</v>
       </c>
       <c r="D2601" t="s">
         <v>2603</v>
@@ -45728,7 +45728,7 @@
         <v>9</v>
       </c>
       <c r="C2602">
-        <v>5410</v>
+        <v>5510</v>
       </c>
       <c r="D2602" t="s">
         <v>2604</v>
@@ -45742,7 +45742,7 @@
         <v>10</v>
       </c>
       <c r="C2603">
-        <v>5390</v>
+        <v>5490</v>
       </c>
       <c r="D2603" t="s">
         <v>2605</v>
@@ -45756,7 +45756,7 @@
         <v>11</v>
       </c>
       <c r="C2604">
-        <v>5360</v>
+        <v>5470</v>
       </c>
       <c r="D2604" t="s">
         <v>2606</v>
@@ -45770,7 +45770,7 @@
         <v>12</v>
       </c>
       <c r="C2605">
-        <v>5340</v>
+        <v>5450</v>
       </c>
       <c r="D2605" t="s">
         <v>2607</v>
@@ -45784,7 +45784,7 @@
         <v>13</v>
       </c>
       <c r="C2606">
-        <v>5320</v>
+        <v>5430</v>
       </c>
       <c r="D2606" t="s">
         <v>2608</v>
@@ -45798,7 +45798,7 @@
         <v>14</v>
       </c>
       <c r="C2607">
-        <v>5300</v>
+        <v>5400</v>
       </c>
       <c r="D2607" t="s">
         <v>2609</v>
@@ -45812,7 +45812,7 @@
         <v>15</v>
       </c>
       <c r="C2608">
-        <v>5290</v>
+        <v>5410</v>
       </c>
       <c r="D2608" t="s">
         <v>2610</v>
@@ -45826,7 +45826,7 @@
         <v>16</v>
       </c>
       <c r="C2609">
-        <v>5290</v>
+        <v>5410</v>
       </c>
       <c r="D2609" t="s">
         <v>2611</v>
@@ -45840,7 +45840,7 @@
         <v>17</v>
       </c>
       <c r="C2610">
-        <v>5300</v>
+        <v>5420</v>
       </c>
       <c r="D2610" t="s">
         <v>2612</v>
@@ -45854,7 +45854,7 @@
         <v>18</v>
       </c>
       <c r="C2611">
-        <v>5310</v>
+        <v>5430</v>
       </c>
       <c r="D2611" t="s">
         <v>2613</v>
@@ -45868,7 +45868,7 @@
         <v>19</v>
       </c>
       <c r="C2612">
-        <v>5340</v>
+        <v>5450</v>
       </c>
       <c r="D2612" t="s">
         <v>2614</v>
@@ -45882,7 +45882,7 @@
         <v>20</v>
       </c>
       <c r="C2613">
-        <v>5380</v>
+        <v>5470</v>
       </c>
       <c r="D2613" t="s">
         <v>2615</v>
@@ -45896,7 +45896,7 @@
         <v>21</v>
       </c>
       <c r="C2614">
-        <v>5420</v>
+        <v>5500</v>
       </c>
       <c r="D2614" t="s">
         <v>2616</v>
@@ -45910,7 +45910,7 @@
         <v>22</v>
       </c>
       <c r="C2615">
-        <v>5450</v>
+        <v>5530</v>
       </c>
       <c r="D2615" t="s">
         <v>2617</v>
@@ -45924,7 +45924,7 @@
         <v>23</v>
       </c>
       <c r="C2616">
-        <v>5460</v>
+        <v>5550</v>
       </c>
       <c r="D2616" t="s">
         <v>2618</v>
@@ -45938,7 +45938,7 @@
         <v>24</v>
       </c>
       <c r="C2617">
-        <v>5450</v>
+        <v>5560</v>
       </c>
       <c r="D2617" t="s">
         <v>2619</v>
@@ -45952,7 +45952,7 @@
         <v>25</v>
       </c>
       <c r="C2618">
-        <v>5430</v>
+        <v>5580</v>
       </c>
       <c r="D2618" t="s">
         <v>2620</v>
@@ -45966,7 +45966,7 @@
         <v>26</v>
       </c>
       <c r="C2619">
-        <v>5430</v>
+        <v>5600</v>
       </c>
       <c r="D2619" t="s">
         <v>2621</v>
@@ -45980,7 +45980,7 @@
         <v>27</v>
       </c>
       <c r="C2620">
-        <v>5450</v>
+        <v>5650</v>
       </c>
       <c r="D2620" t="s">
         <v>2622</v>
@@ -45994,7 +45994,7 @@
         <v>28</v>
       </c>
       <c r="C2621">
-        <v>5500</v>
+        <v>5710</v>
       </c>
       <c r="D2621" t="s">
         <v>2623</v>
@@ -46008,7 +46008,7 @@
         <v>29</v>
       </c>
       <c r="C2622">
-        <v>5570</v>
+        <v>5780</v>
       </c>
       <c r="D2622" t="s">
         <v>2624</v>
@@ -46022,7 +46022,7 @@
         <v>30</v>
       </c>
       <c r="C2623">
-        <v>5620</v>
+        <v>5860</v>
       </c>
       <c r="D2623" t="s">
         <v>2625</v>
@@ -46036,7 +46036,7 @@
         <v>31</v>
       </c>
       <c r="C2624">
-        <v>5660</v>
+        <v>5940</v>
       </c>
       <c r="D2624" t="s">
         <v>2626</v>
@@ -46050,7 +46050,7 @@
         <v>32</v>
       </c>
       <c r="C2625">
-        <v>5690</v>
+        <v>6030</v>
       </c>
       <c r="D2625" t="s">
         <v>2627</v>
@@ -46064,7 +46064,7 @@
         <v>33</v>
       </c>
       <c r="C2626">
-        <v>5700</v>
+        <v>6110</v>
       </c>
       <c r="D2626" t="s">
         <v>2628</v>
@@ -46078,7 +46078,7 @@
         <v>34</v>
       </c>
       <c r="C2627">
-        <v>5700</v>
+        <v>6180</v>
       </c>
       <c r="D2627" t="s">
         <v>2629</v>
@@ -46092,7 +46092,7 @@
         <v>35</v>
       </c>
       <c r="C2628">
-        <v>5710</v>
+        <v>6230</v>
       </c>
       <c r="D2628" t="s">
         <v>2630</v>
@@ -46106,7 +46106,7 @@
         <v>36</v>
       </c>
       <c r="C2629">
-        <v>5710</v>
+        <v>6270</v>
       </c>
       <c r="D2629" t="s">
         <v>2631</v>
@@ -46120,7 +46120,7 @@
         <v>37</v>
       </c>
       <c r="C2630">
-        <v>5710</v>
+        <v>6290</v>
       </c>
       <c r="D2630" t="s">
         <v>2632</v>
@@ -46134,7 +46134,7 @@
         <v>38</v>
       </c>
       <c r="C2631">
-        <v>5700</v>
+        <v>6300</v>
       </c>
       <c r="D2631" t="s">
         <v>2633</v>
@@ -46148,7 +46148,7 @@
         <v>39</v>
       </c>
       <c r="C2632">
-        <v>5680</v>
+        <v>6300</v>
       </c>
       <c r="D2632" t="s">
         <v>2634</v>
@@ -46162,7 +46162,7 @@
         <v>40</v>
       </c>
       <c r="C2633">
-        <v>5660</v>
+        <v>6300</v>
       </c>
       <c r="D2633" t="s">
         <v>2635</v>
@@ -46176,7 +46176,7 @@
         <v>41</v>
       </c>
       <c r="C2634">
-        <v>5620</v>
+        <v>6300</v>
       </c>
       <c r="D2634" t="s">
         <v>2636</v>
@@ -46190,7 +46190,7 @@
         <v>42</v>
       </c>
       <c r="C2635">
-        <v>5580</v>
+        <v>6300</v>
       </c>
       <c r="D2635" t="s">
         <v>2637</v>
@@ -46204,7 +46204,7 @@
         <v>43</v>
       </c>
       <c r="C2636">
-        <v>5540</v>
+        <v>6300</v>
       </c>
       <c r="D2636" t="s">
         <v>2638</v>
@@ -46218,7 +46218,7 @@
         <v>44</v>
       </c>
       <c r="C2637">
-        <v>5490</v>
+        <v>6290</v>
       </c>
       <c r="D2637" t="s">
         <v>2639</v>
@@ -46232,7 +46232,7 @@
         <v>45</v>
       </c>
       <c r="C2638">
-        <v>5450</v>
+        <v>6260</v>
       </c>
       <c r="D2638" t="s">
         <v>2640</v>
@@ -46246,7 +46246,7 @@
         <v>46</v>
       </c>
       <c r="C2639">
-        <v>5400</v>
+        <v>6230</v>
       </c>
       <c r="D2639" t="s">
         <v>2641</v>
@@ -46260,7 +46260,7 @@
         <v>47</v>
       </c>
       <c r="C2640">
-        <v>5360</v>
+        <v>6210</v>
       </c>
       <c r="D2640" t="s">
         <v>2642</v>
@@ -46274,7 +46274,7 @@
         <v>48</v>
       </c>
       <c r="C2641">
-        <v>5320</v>
+        <v>6200</v>
       </c>
       <c r="D2641" t="s">
         <v>2643</v>
@@ -46288,7 +46288,7 @@
         <v>49</v>
       </c>
       <c r="C2642">
-        <v>5280</v>
+        <v>6190</v>
       </c>
       <c r="D2642" t="s">
         <v>2644</v>
@@ -46302,7 +46302,7 @@
         <v>50</v>
       </c>
       <c r="C2643">
-        <v>5250</v>
+        <v>6180</v>
       </c>
       <c r="D2643" t="s">
         <v>2645</v>
@@ -46316,7 +46316,7 @@
         <v>51</v>
       </c>
       <c r="C2644">
-        <v>5230</v>
+        <v>6170</v>
       </c>
       <c r="D2644" t="s">
         <v>2646</v>
@@ -46330,7 +46330,7 @@
         <v>52</v>
       </c>
       <c r="C2645">
-        <v>5220</v>
+        <v>6160</v>
       </c>
       <c r="D2645" t="s">
         <v>2647</v>
@@ -46344,7 +46344,7 @@
         <v>53</v>
       </c>
       <c r="C2646">
-        <v>5220</v>
+        <v>6150</v>
       </c>
       <c r="D2646" t="s">
         <v>2648</v>
@@ -46358,7 +46358,7 @@
         <v>54</v>
       </c>
       <c r="C2647">
-        <v>5220</v>
+        <v>6140</v>
       </c>
       <c r="D2647" t="s">
         <v>2649</v>
@@ -46372,7 +46372,7 @@
         <v>55</v>
       </c>
       <c r="C2648">
-        <v>5240</v>
+        <v>6140</v>
       </c>
       <c r="D2648" t="s">
         <v>2650</v>
@@ -46386,7 +46386,7 @@
         <v>56</v>
       </c>
       <c r="C2649">
-        <v>5260</v>
+        <v>6140</v>
       </c>
       <c r="D2649" t="s">
         <v>2651</v>
@@ -46400,7 +46400,7 @@
         <v>57</v>
       </c>
       <c r="C2650">
-        <v>5290</v>
+        <v>6140</v>
       </c>
       <c r="D2650" t="s">
         <v>2652</v>
@@ -46414,7 +46414,7 @@
         <v>58</v>
       </c>
       <c r="C2651">
-        <v>5320</v>
+        <v>6140</v>
       </c>
       <c r="D2651" t="s">
         <v>2653</v>
@@ -46428,7 +46428,7 @@
         <v>59</v>
       </c>
       <c r="C2652">
-        <v>5350</v>
+        <v>6140</v>
       </c>
       <c r="D2652" t="s">
         <v>2654</v>
@@ -46442,7 +46442,7 @@
         <v>60</v>
       </c>
       <c r="C2653">
-        <v>5370</v>
+        <v>6140</v>
       </c>
       <c r="D2653" t="s">
         <v>2655</v>
@@ -46456,7 +46456,7 @@
         <v>61</v>
       </c>
       <c r="C2654">
-        <v>5390</v>
+        <v>6140</v>
       </c>
       <c r="D2654" t="s">
         <v>2656</v>
@@ -46470,7 +46470,7 @@
         <v>62</v>
       </c>
       <c r="C2655">
-        <v>5420</v>
+        <v>6160</v>
       </c>
       <c r="D2655" t="s">
         <v>2657</v>
@@ -46484,7 +46484,7 @@
         <v>63</v>
       </c>
       <c r="C2656">
-        <v>5480</v>
+        <v>6180</v>
       </c>
       <c r="D2656" t="s">
         <v>2658</v>
@@ -46498,7 +46498,7 @@
         <v>64</v>
       </c>
       <c r="C2657">
-        <v>5560</v>
+        <v>6220</v>
       </c>
       <c r="D2657" t="s">
         <v>2659</v>
@@ -46512,7 +46512,7 @@
         <v>65</v>
       </c>
       <c r="C2658">
-        <v>5660</v>
+        <v>6280</v>
       </c>
       <c r="D2658" t="s">
         <v>2660</v>
@@ -46526,7 +46526,7 @@
         <v>66</v>
       </c>
       <c r="C2659">
-        <v>5760</v>
+        <v>6340</v>
       </c>
       <c r="D2659" t="s">
         <v>2661</v>
@@ -46540,7 +46540,7 @@
         <v>67</v>
       </c>
       <c r="C2660">
-        <v>5870</v>
+        <v>6410</v>
       </c>
       <c r="D2660" t="s">
         <v>2662</v>
@@ -46554,7 +46554,7 @@
         <v>68</v>
       </c>
       <c r="C2661">
-        <v>5970</v>
+        <v>6490</v>
       </c>
       <c r="D2661" t="s">
         <v>2663</v>
@@ -46568,7 +46568,7 @@
         <v>69</v>
       </c>
       <c r="C2662">
-        <v>6080</v>
+        <v>6580</v>
       </c>
       <c r="D2662" t="s">
         <v>2664</v>
@@ -46582,7 +46582,7 @@
         <v>70</v>
       </c>
       <c r="C2663">
-        <v>6180</v>
+        <v>6660</v>
       </c>
       <c r="D2663" t="s">
         <v>2665</v>
@@ -46596,7 +46596,7 @@
         <v>71</v>
       </c>
       <c r="C2664">
-        <v>6260</v>
+        <v>6740</v>
       </c>
       <c r="D2664" t="s">
         <v>2666</v>
@@ -46610,7 +46610,7 @@
         <v>72</v>
       </c>
       <c r="C2665">
-        <v>6340</v>
+        <v>6800</v>
       </c>
       <c r="D2665" t="s">
         <v>2667</v>
@@ -46624,7 +46624,7 @@
         <v>73</v>
       </c>
       <c r="C2666">
-        <v>6410</v>
+        <v>6860</v>
       </c>
       <c r="D2666" t="s">
         <v>2668</v>
@@ -46638,7 +46638,7 @@
         <v>74</v>
       </c>
       <c r="C2667">
-        <v>6500</v>
+        <v>6900</v>
       </c>
       <c r="D2667" t="s">
         <v>2669</v>
@@ -46652,7 +46652,7 @@
         <v>75</v>
       </c>
       <c r="C2668">
-        <v>6610</v>
+        <v>6960</v>
       </c>
       <c r="D2668" t="s">
         <v>2670</v>
@@ -46666,7 +46666,7 @@
         <v>76</v>
       </c>
       <c r="C2669">
-        <v>6760</v>
+        <v>6980</v>
       </c>
       <c r="D2669" t="s">
         <v>2671</v>
@@ -46680,7 +46680,7 @@
         <v>77</v>
       </c>
       <c r="C2670">
-        <v>6910</v>
+        <v>7050</v>
       </c>
       <c r="D2670" t="s">
         <v>2672</v>
@@ -46694,7 +46694,7 @@
         <v>78</v>
       </c>
       <c r="C2671">
-        <v>7020</v>
+        <v>7090</v>
       </c>
       <c r="D2671" t="s">
         <v>2673</v>
@@ -46708,7 +46708,7 @@
         <v>79</v>
       </c>
       <c r="C2672">
-        <v>7080</v>
+        <v>7100</v>
       </c>
       <c r="D2672" t="s">
         <v>2674</v>
@@ -46722,7 +46722,7 @@
         <v>80</v>
       </c>
       <c r="C2673">
-        <v>7080</v>
+        <v>7140</v>
       </c>
       <c r="D2673" t="s">
         <v>2675</v>
@@ -46736,7 +46736,7 @@
         <v>81</v>
       </c>
       <c r="C2674">
-        <v>7030</v>
+        <v>7150</v>
       </c>
       <c r="D2674" t="s">
         <v>2676</v>
@@ -46750,7 +46750,7 @@
         <v>82</v>
       </c>
       <c r="C2675">
-        <v>6970</v>
+        <v>7130</v>
       </c>
       <c r="D2675" t="s">
         <v>2677</v>
@@ -46764,7 +46764,7 @@
         <v>83</v>
       </c>
       <c r="C2676">
-        <v>6920</v>
+        <v>7110</v>
       </c>
       <c r="D2676" t="s">
         <v>2678</v>
@@ -46778,7 +46778,7 @@
         <v>84</v>
       </c>
       <c r="C2677">
-        <v>6870</v>
+        <v>7080</v>
       </c>
       <c r="D2677" t="s">
         <v>2679</v>
@@ -46792,7 +46792,7 @@
         <v>85</v>
       </c>
       <c r="C2678">
-        <v>6820</v>
+        <v>6990</v>
       </c>
       <c r="D2678" t="s">
         <v>2680</v>
@@ -46806,7 +46806,7 @@
         <v>86</v>
       </c>
       <c r="C2679">
-        <v>6740</v>
+        <v>6890</v>
       </c>
       <c r="D2679" t="s">
         <v>2681</v>
@@ -46820,7 +46820,7 @@
         <v>87</v>
       </c>
       <c r="C2680">
-        <v>6640</v>
+        <v>6790</v>
       </c>
       <c r="D2680" t="s">
         <v>2682</v>
@@ -46834,7 +46834,7 @@
         <v>88</v>
       </c>
       <c r="C2681">
-        <v>6500</v>
+        <v>6670</v>
       </c>
       <c r="D2681" t="s">
         <v>2683</v>
@@ -46848,7 +46848,7 @@
         <v>89</v>
       </c>
       <c r="C2682">
-        <v>6350</v>
+        <v>6550</v>
       </c>
       <c r="D2682" t="s">
         <v>2684</v>
@@ -46862,7 +46862,7 @@
         <v>90</v>
       </c>
       <c r="C2683">
-        <v>6200</v>
+        <v>6430</v>
       </c>
       <c r="D2683" t="s">
         <v>2685</v>
@@ -46876,7 +46876,7 @@
         <v>91</v>
       </c>
       <c r="C2684">
-        <v>6060</v>
+        <v>6300</v>
       </c>
       <c r="D2684" t="s">
         <v>2686</v>
@@ -46890,7 +46890,7 @@
         <v>92</v>
       </c>
       <c r="C2685">
-        <v>5940</v>
+        <v>6180</v>
       </c>
       <c r="D2685" t="s">
         <v>2687</v>
@@ -46904,7 +46904,7 @@
         <v>93</v>
       </c>
       <c r="C2686">
-        <v>5830</v>
+        <v>6050</v>
       </c>
       <c r="D2686" t="s">
         <v>2688</v>
@@ -46918,7 +46918,7 @@
         <v>94</v>
       </c>
       <c r="C2687">
-        <v>5720</v>
+        <v>5930</v>
       </c>
       <c r="D2687" t="s">
         <v>2689</v>
@@ -46932,7 +46932,7 @@
         <v>95</v>
       </c>
       <c r="C2688">
-        <v>5630</v>
+        <v>5830</v>
       </c>
       <c r="D2688" t="s">
         <v>2690</v>
@@ -46946,7 +46946,7 @@
         <v>96</v>
       </c>
       <c r="C2689">
-        <v>5540</v>
+        <v>5730</v>
       </c>
       <c r="D2689" t="s">
         <v>2691</v>
@@ -46960,7 +46960,7 @@
         <v>1</v>
       </c>
       <c r="C2690">
-        <v>5460</v>
+        <v>5610</v>
       </c>
       <c r="D2690" t="s">
         <v>2692</v>
@@ -46974,7 +46974,7 @@
         <v>2</v>
       </c>
       <c r="C2691">
-        <v>5390</v>
+        <v>5530</v>
       </c>
       <c r="D2691" t="s">
         <v>2693</v>
@@ -46988,7 +46988,7 @@
         <v>3</v>
       </c>
       <c r="C2692">
-        <v>5320</v>
+        <v>5460</v>
       </c>
       <c r="D2692" t="s">
         <v>2694</v>
@@ -47002,7 +47002,7 @@
         <v>4</v>
       </c>
       <c r="C2693">
-        <v>5260</v>
+        <v>5390</v>
       </c>
       <c r="D2693" t="s">
         <v>2695</v>
@@ -47016,7 +47016,7 @@
         <v>5</v>
       </c>
       <c r="C2694">
-        <v>5210</v>
+        <v>5330</v>
       </c>
       <c r="D2694" t="s">
         <v>2696</v>
@@ -47030,7 +47030,7 @@
         <v>6</v>
       </c>
       <c r="C2695">
-        <v>5160</v>
+        <v>5280</v>
       </c>
       <c r="D2695" t="s">
         <v>2697</v>
@@ -47044,7 +47044,7 @@
         <v>7</v>
       </c>
       <c r="C2696">
-        <v>5120</v>
+        <v>5240</v>
       </c>
       <c r="D2696" t="s">
         <v>2698</v>
@@ -47058,7 +47058,7 @@
         <v>8</v>
       </c>
       <c r="C2697">
-        <v>5090</v>
+        <v>5210</v>
       </c>
       <c r="D2697" t="s">
         <v>2699</v>
@@ -47072,7 +47072,7 @@
         <v>9</v>
       </c>
       <c r="C2698">
-        <v>5070</v>
+        <v>5180</v>
       </c>
       <c r="D2698" t="s">
         <v>2700</v>
@@ -47086,7 +47086,7 @@
         <v>10</v>
       </c>
       <c r="C2699">
-        <v>5050</v>
+        <v>5110</v>
       </c>
       <c r="D2699" t="s">
         <v>2701</v>
@@ -47100,7 +47100,7 @@
         <v>11</v>
       </c>
       <c r="C2700">
-        <v>5020</v>
+        <v>5060</v>
       </c>
       <c r="D2700" t="s">
         <v>2702</v>
@@ -47128,7 +47128,7 @@
         <v>17</v>
       </c>
       <c r="C2702">
-        <v>4980</v>
+        <v>5000</v>
       </c>
       <c r="D2702" t="s">
         <v>2704</v>
@@ -47142,7 +47142,7 @@
         <v>18</v>
       </c>
       <c r="C2703">
-        <v>4970</v>
+        <v>5020</v>
       </c>
       <c r="D2703" t="s">
         <v>2705</v>
@@ -47156,7 +47156,7 @@
         <v>19</v>
       </c>
       <c r="C2704">
-        <v>4970</v>
+        <v>5050</v>
       </c>
       <c r="D2704" t="s">
         <v>2706</v>
@@ -47170,7 +47170,7 @@
         <v>20</v>
       </c>
       <c r="C2705">
-        <v>4980</v>
+        <v>5080</v>
       </c>
       <c r="D2705" t="s">
         <v>2707</v>
@@ -47184,7 +47184,7 @@
         <v>21</v>
       </c>
       <c r="C2706">
-        <v>5000</v>
+        <v>5120</v>
       </c>
       <c r="D2706" t="s">
         <v>2708</v>
@@ -47198,7 +47198,7 @@
         <v>22</v>
       </c>
       <c r="C2707">
-        <v>5020</v>
+        <v>5140</v>
       </c>
       <c r="D2707" t="s">
         <v>2709</v>
@@ -47212,7 +47212,7 @@
         <v>23</v>
       </c>
       <c r="C2708">
-        <v>5050</v>
+        <v>5160</v>
       </c>
       <c r="D2708" t="s">
         <v>2710</v>
@@ -47226,7 +47226,7 @@
         <v>24</v>
       </c>
       <c r="C2709">
-        <v>5070</v>
+        <v>5180</v>
       </c>
       <c r="D2709" t="s">
         <v>2711</v>
@@ -47240,7 +47240,7 @@
         <v>25</v>
       </c>
       <c r="C2710">
-        <v>5090</v>
+        <v>5190</v>
       </c>
       <c r="D2710" t="s">
         <v>2712</v>
@@ -47254,7 +47254,7 @@
         <v>26</v>
       </c>
       <c r="C2711">
-        <v>5100</v>
+        <v>5210</v>
       </c>
       <c r="D2711" t="s">
         <v>2713</v>
@@ -47268,7 +47268,7 @@
         <v>27</v>
       </c>
       <c r="C2712">
-        <v>5100</v>
+        <v>5220</v>
       </c>
       <c r="D2712" t="s">
         <v>2714</v>
@@ -47282,7 +47282,7 @@
         <v>28</v>
       </c>
       <c r="C2713">
-        <v>5090</v>
+        <v>5240</v>
       </c>
       <c r="D2713" t="s">
         <v>2715</v>
@@ -47296,7 +47296,7 @@
         <v>29</v>
       </c>
       <c r="C2714">
-        <v>5080</v>
+        <v>5250</v>
       </c>
       <c r="D2714" t="s">
         <v>2716</v>
@@ -47310,7 +47310,7 @@
         <v>30</v>
       </c>
       <c r="C2715">
-        <v>5080</v>
+        <v>5280</v>
       </c>
       <c r="D2715" t="s">
         <v>2717</v>
@@ -47324,7 +47324,7 @@
         <v>31</v>
       </c>
       <c r="C2716">
-        <v>5110</v>
+        <v>5320</v>
       </c>
       <c r="D2716" t="s">
         <v>2718</v>
@@ -47338,7 +47338,7 @@
         <v>32</v>
       </c>
       <c r="C2717">
-        <v>5160</v>
+        <v>5380</v>
       </c>
       <c r="D2717" t="s">
         <v>2719</v>
@@ -47352,7 +47352,7 @@
         <v>33</v>
       </c>
       <c r="C2718">
-        <v>5230</v>
+        <v>5450</v>
       </c>
       <c r="D2718" t="s">
         <v>2720</v>
@@ -47366,7 +47366,7 @@
         <v>34</v>
       </c>
       <c r="C2719">
-        <v>5280</v>
+        <v>5470</v>
       </c>
       <c r="D2719" t="s">
         <v>2721</v>
@@ -47380,7 +47380,7 @@
         <v>35</v>
       </c>
       <c r="C2720">
-        <v>5300</v>
+        <v>5480</v>
       </c>
       <c r="D2720" t="s">
         <v>2722</v>
@@ -47394,7 +47394,7 @@
         <v>36</v>
       </c>
       <c r="C2721">
-        <v>5290</v>
+        <v>5490</v>
       </c>
       <c r="D2721" t="s">
         <v>2723</v>
@@ -47408,7 +47408,7 @@
         <v>37</v>
       </c>
       <c r="C2722">
-        <v>5250</v>
+        <v>5500</v>
       </c>
       <c r="D2722" t="s">
         <v>2724</v>
@@ -47422,7 +47422,7 @@
         <v>38</v>
       </c>
       <c r="C2723">
-        <v>5210</v>
+        <v>5520</v>
       </c>
       <c r="D2723" t="s">
         <v>2725</v>
@@ -47436,7 +47436,7 @@
         <v>39</v>
       </c>
       <c r="C2724">
-        <v>5180</v>
+        <v>5550</v>
       </c>
       <c r="D2724" t="s">
         <v>2726</v>
@@ -47450,7 +47450,7 @@
         <v>40</v>
       </c>
       <c r="C2725">
-        <v>5150</v>
+        <v>5550</v>
       </c>
       <c r="D2725" t="s">
         <v>2727</v>
@@ -47464,7 +47464,7 @@
         <v>41</v>
       </c>
       <c r="C2726">
-        <v>5120</v>
+        <v>5550</v>
       </c>
       <c r="D2726" t="s">
         <v>2728</v>
@@ -47478,7 +47478,7 @@
         <v>42</v>
       </c>
       <c r="C2727">
-        <v>5090</v>
+        <v>5530</v>
       </c>
       <c r="D2727" t="s">
         <v>2729</v>
@@ -47492,7 +47492,7 @@
         <v>43</v>
       </c>
       <c r="C2728">
-        <v>5050</v>
+        <v>5520</v>
       </c>
       <c r="D2728" t="s">
         <v>2730</v>
@@ -47506,7 +47506,7 @@
         <v>44</v>
       </c>
       <c r="C2729">
-        <v>5000</v>
+        <v>5500</v>
       </c>
       <c r="D2729" t="s">
         <v>2731</v>
@@ -47520,7 +47520,7 @@
         <v>45</v>
       </c>
       <c r="C2730">
-        <v>4950</v>
+        <v>5480</v>
       </c>
       <c r="D2730" t="s">
         <v>2732</v>
@@ -47534,7 +47534,7 @@
         <v>46</v>
       </c>
       <c r="C2731">
-        <v>4900</v>
+        <v>5490</v>
       </c>
       <c r="D2731" t="s">
         <v>2733</v>
@@ -47548,7 +47548,7 @@
         <v>47</v>
       </c>
       <c r="C2732">
-        <v>4850</v>
+        <v>5460</v>
       </c>
       <c r="D2732" t="s">
         <v>2734</v>
@@ -47562,7 +47562,7 @@
         <v>48</v>
       </c>
       <c r="C2733">
-        <v>4810</v>
+        <v>5410</v>
       </c>
       <c r="D2733" t="s">
         <v>2735</v>
@@ -47576,7 +47576,7 @@
         <v>49</v>
       </c>
       <c r="C2734">
-        <v>4780</v>
+        <v>5370</v>
       </c>
       <c r="D2734" t="s">
         <v>2736</v>
@@ -47590,7 +47590,7 @@
         <v>50</v>
       </c>
       <c r="C2735">
-        <v>4750</v>
+        <v>5330</v>
       </c>
       <c r="D2735" t="s">
         <v>2737</v>
@@ -47604,7 +47604,7 @@
         <v>51</v>
       </c>
       <c r="C2736">
-        <v>4730</v>
+        <v>5310</v>
       </c>
       <c r="D2736" t="s">
         <v>2738</v>
@@ -47618,7 +47618,7 @@
         <v>52</v>
       </c>
       <c r="C2737">
-        <v>4720</v>
+        <v>5310</v>
       </c>
       <c r="D2737" t="s">
         <v>2739</v>
@@ -47632,7 +47632,7 @@
         <v>53</v>
       </c>
       <c r="C2738">
-        <v>4720</v>
+        <v>5330</v>
       </c>
       <c r="D2738" t="s">
         <v>2740</v>
@@ -47646,7 +47646,7 @@
         <v>54</v>
       </c>
       <c r="C2739">
-        <v>4710</v>
+        <v>5330</v>
       </c>
       <c r="D2739" t="s">
         <v>2741</v>
@@ -47660,7 +47660,7 @@
         <v>55</v>
       </c>
       <c r="C2740">
-        <v>4690</v>
+        <v>5310</v>
       </c>
       <c r="D2740" t="s">
         <v>2742</v>
@@ -47674,7 +47674,7 @@
         <v>56</v>
       </c>
       <c r="C2741">
-        <v>4660</v>
+        <v>5280</v>
       </c>
       <c r="D2741" t="s">
         <v>2743</v>
@@ -47688,7 +47688,7 @@
         <v>57</v>
       </c>
       <c r="C2742">
-        <v>4630</v>
+        <v>5240</v>
       </c>
       <c r="D2742" t="s">
         <v>2744</v>
@@ -47702,7 +47702,7 @@
         <v>58</v>
       </c>
       <c r="C2743">
-        <v>4610</v>
+        <v>5210</v>
       </c>
       <c r="D2743" t="s">
         <v>2745</v>
@@ -47716,7 +47716,7 @@
         <v>59</v>
       </c>
       <c r="C2744">
-        <v>4600</v>
+        <v>5210</v>
       </c>
       <c r="D2744" t="s">
         <v>2746</v>
@@ -47730,7 +47730,7 @@
         <v>60</v>
       </c>
       <c r="C2745">
-        <v>4590</v>
+        <v>5230</v>
       </c>
       <c r="D2745" t="s">
         <v>2747</v>
@@ -47744,7 +47744,7 @@
         <v>61</v>
       </c>
       <c r="C2746">
-        <v>4610</v>
+        <v>5270</v>
       </c>
       <c r="D2746" t="s">
         <v>2748</v>
@@ -47758,7 +47758,7 @@
         <v>62</v>
       </c>
       <c r="C2747">
-        <v>4630</v>
+        <v>5320</v>
       </c>
       <c r="D2747" t="s">
         <v>2749</v>
@@ -47772,7 +47772,7 @@
         <v>63</v>
       </c>
       <c r="C2748">
-        <v>4680</v>
+        <v>5370</v>
       </c>
       <c r="D2748" t="s">
         <v>2750</v>
@@ -47786,7 +47786,7 @@
         <v>64</v>
       </c>
       <c r="C2749">
-        <v>4750</v>
+        <v>5420</v>
       </c>
       <c r="D2749" t="s">
         <v>2751</v>
@@ -47800,7 +47800,7 @@
         <v>65</v>
       </c>
       <c r="C2750">
-        <v>4830</v>
+        <v>5480</v>
       </c>
       <c r="D2750" t="s">
         <v>2752</v>
@@ -47814,7 +47814,7 @@
         <v>66</v>
       </c>
       <c r="C2751">
-        <v>4920</v>
+        <v>5550</v>
       </c>
       <c r="D2751" t="s">
         <v>2753</v>
@@ -47828,7 +47828,7 @@
         <v>67</v>
       </c>
       <c r="C2752">
-        <v>5010</v>
+        <v>5620</v>
       </c>
       <c r="D2752" t="s">
         <v>2754</v>
@@ -47842,7 +47842,7 @@
         <v>68</v>
       </c>
       <c r="C2753">
-        <v>5100</v>
+        <v>5690</v>
       </c>
       <c r="D2753" t="s">
         <v>2755</v>
@@ -47856,7 +47856,7 @@
         <v>69</v>
       </c>
       <c r="C2754">
-        <v>5190</v>
+        <v>5770</v>
       </c>
       <c r="D2754" t="s">
         <v>2756</v>
@@ -47870,7 +47870,7 @@
         <v>70</v>
       </c>
       <c r="C2755">
-        <v>5280</v>
+        <v>5840</v>
       </c>
       <c r="D2755" t="s">
         <v>2757</v>
@@ -47884,7 +47884,7 @@
         <v>71</v>
       </c>
       <c r="C2756">
-        <v>5380</v>
+        <v>5910</v>
       </c>
       <c r="D2756" t="s">
         <v>2758</v>
@@ -47898,7 +47898,7 @@
         <v>72</v>
       </c>
       <c r="C2757">
-        <v>5480</v>
+        <v>5980</v>
       </c>
       <c r="D2757" t="s">
         <v>2759</v>
@@ -47912,7 +47912,7 @@
         <v>73</v>
       </c>
       <c r="C2758">
-        <v>5590</v>
+        <v>6040</v>
       </c>
       <c r="D2758" t="s">
         <v>2760</v>
@@ -47926,7 +47926,7 @@
         <v>74</v>
       </c>
       <c r="C2759">
-        <v>5690</v>
+        <v>6110</v>
       </c>
       <c r="D2759" t="s">
         <v>2761</v>
@@ -47940,7 +47940,7 @@
         <v>75</v>
       </c>
       <c r="C2760">
-        <v>5780</v>
+        <v>6180</v>
       </c>
       <c r="D2760" t="s">
         <v>2762</v>
@@ -47954,7 +47954,7 @@
         <v>76</v>
       </c>
       <c r="C2761">
-        <v>5870</v>
+        <v>6260</v>
       </c>
       <c r="D2761" t="s">
         <v>2763</v>
@@ -47968,7 +47968,7 @@
         <v>77</v>
       </c>
       <c r="C2762">
-        <v>5950</v>
+        <v>6340</v>
       </c>
       <c r="D2762" t="s">
         <v>2764</v>
@@ -47982,7 +47982,7 @@
         <v>78</v>
       </c>
       <c r="C2763">
-        <v>6040</v>
+        <v>6420</v>
       </c>
       <c r="D2763" t="s">
         <v>2765</v>
@@ -47996,7 +47996,7 @@
         <v>79</v>
       </c>
       <c r="C2764">
-        <v>6160</v>
+        <v>6500</v>
       </c>
       <c r="D2764" t="s">
         <v>2766</v>
@@ -48010,7 +48010,7 @@
         <v>80</v>
       </c>
       <c r="C2765">
-        <v>6290</v>
+        <v>6550</v>
       </c>
       <c r="D2765" t="s">
         <v>2767</v>
@@ -48024,7 +48024,7 @@
         <v>81</v>
       </c>
       <c r="C2766">
-        <v>6440</v>
+        <v>6580</v>
       </c>
       <c r="D2766" t="s">
         <v>2768</v>
@@ -48038,7 +48038,7 @@
         <v>82</v>
       </c>
       <c r="C2767">
-        <v>6530</v>
+        <v>6590</v>
       </c>
       <c r="D2767" t="s">
         <v>2769</v>
@@ -48052,7 +48052,7 @@
         <v>83</v>
       </c>
       <c r="C2768">
-        <v>6560</v>
+        <v>6600</v>
       </c>
       <c r="D2768" t="s">
         <v>2770</v>
@@ -48066,7 +48066,7 @@
         <v>84</v>
       </c>
       <c r="C2769">
-        <v>6530</v>
+        <v>6600</v>
       </c>
       <c r="D2769" t="s">
         <v>2771</v>
@@ -48080,7 +48080,7 @@
         <v>85</v>
       </c>
       <c r="C2770">
-        <v>6450</v>
+        <v>6580</v>
       </c>
       <c r="D2770" t="s">
         <v>2772</v>
@@ -48094,7 +48094,7 @@
         <v>86</v>
       </c>
       <c r="C2771">
-        <v>6360</v>
+        <v>6520</v>
       </c>
       <c r="D2771" t="s">
         <v>2773</v>
@@ -48108,7 +48108,7 @@
         <v>87</v>
       </c>
       <c r="C2772">
-        <v>6260</v>
+        <v>6420</v>
       </c>
       <c r="D2772" t="s">
         <v>2774</v>
@@ -48122,7 +48122,7 @@
         <v>88</v>
       </c>
       <c r="C2773">
-        <v>6160</v>
+        <v>6320</v>
       </c>
       <c r="D2773" t="s">
         <v>2775</v>
@@ -48136,7 +48136,7 @@
         <v>89</v>
       </c>
       <c r="C2774">
-        <v>6050</v>
+        <v>6210</v>
       </c>
       <c r="D2774" t="s">
         <v>2776</v>
@@ -48150,7 +48150,7 @@
         <v>90</v>
       </c>
       <c r="C2775">
-        <v>5940</v>
+        <v>6090</v>
       </c>
       <c r="D2775" t="s">
         <v>2777</v>
@@ -48164,7 +48164,7 @@
         <v>91</v>
       </c>
       <c r="C2776">
-        <v>5830</v>
+        <v>5970</v>
       </c>
       <c r="D2776" t="s">
         <v>2778</v>
@@ -48178,7 +48178,7 @@
         <v>92</v>
       </c>
       <c r="C2777">
-        <v>5710</v>
+        <v>5860</v>
       </c>
       <c r="D2777" t="s">
         <v>2779</v>
@@ -48192,7 +48192,7 @@
         <v>93</v>
       </c>
       <c r="C2778">
-        <v>5600</v>
+        <v>5740</v>
       </c>
       <c r="D2778" t="s">
         <v>2780</v>
@@ -48206,7 +48206,7 @@
         <v>94</v>
       </c>
       <c r="C2779">
-        <v>5490</v>
+        <v>5640</v>
       </c>
       <c r="D2779" t="s">
         <v>2781</v>
@@ -48220,7 +48220,7 @@
         <v>95</v>
       </c>
       <c r="C2780">
-        <v>5400</v>
+        <v>5550</v>
       </c>
       <c r="D2780" t="s">
         <v>2782</v>
@@ -48234,7 +48234,7 @@
         <v>96</v>
       </c>
       <c r="C2781">
-        <v>5320</v>
+        <v>5470</v>
       </c>
       <c r="D2781" t="s">
         <v>2783</v>
@@ -48248,7 +48248,7 @@
         <v>1</v>
       </c>
       <c r="C2782">
-        <v>5230</v>
+        <v>5420</v>
       </c>
       <c r="D2782" t="s">
         <v>2784</v>
@@ -48262,7 +48262,7 @@
         <v>2</v>
       </c>
       <c r="C2783">
-        <v>5160</v>
+        <v>5360</v>
       </c>
       <c r="D2783" t="s">
         <v>2785</v>
@@ -48276,7 +48276,7 @@
         <v>3</v>
       </c>
       <c r="C2784">
-        <v>5110</v>
+        <v>5300</v>
       </c>
       <c r="D2784" t="s">
         <v>2786</v>
@@ -48290,7 +48290,7 @@
         <v>4</v>
       </c>
       <c r="C2785">
-        <v>5060</v>
+        <v>5250</v>
       </c>
       <c r="D2785" t="s">
         <v>2787</v>
@@ -48304,7 +48304,7 @@
         <v>5</v>
       </c>
       <c r="C2786">
-        <v>5020</v>
+        <v>5200</v>
       </c>
       <c r="D2786" t="s">
         <v>2788</v>
@@ -48318,7 +48318,7 @@
         <v>6</v>
       </c>
       <c r="C2787">
-        <v>4990</v>
+        <v>5160</v>
       </c>
       <c r="D2787" t="s">
         <v>2789</v>
@@ -48332,7 +48332,7 @@
         <v>7</v>
       </c>
       <c r="C2788">
-        <v>4960</v>
+        <v>5130</v>
       </c>
       <c r="D2788" t="s">
         <v>2790</v>
@@ -48346,7 +48346,7 @@
         <v>8</v>
       </c>
       <c r="C2789">
-        <v>4930</v>
+        <v>5110</v>
       </c>
       <c r="D2789" t="s">
         <v>2791</v>
@@ -48360,7 +48360,7 @@
         <v>9</v>
       </c>
       <c r="C2790">
-        <v>4910</v>
+        <v>5100</v>
       </c>
       <c r="D2790" t="s">
         <v>2792</v>
@@ -48374,7 +48374,7 @@
         <v>10</v>
       </c>
       <c r="C2791">
-        <v>4900</v>
+        <v>5080</v>
       </c>
       <c r="D2791" t="s">
         <v>2793</v>
@@ -48388,7 +48388,7 @@
         <v>11</v>
       </c>
       <c r="C2792">
-        <v>4890</v>
+        <v>5050</v>
       </c>
       <c r="D2792" t="s">
         <v>2794</v>
@@ -48402,7 +48402,7 @@
         <v>12</v>
       </c>
       <c r="C2793">
-        <v>4890</v>
+        <v>5020</v>
       </c>
       <c r="D2793" t="s">
         <v>2795</v>
@@ -48416,7 +48416,7 @@
         <v>13</v>
       </c>
       <c r="C2794">
-        <v>4890</v>
+        <v>5010</v>
       </c>
       <c r="D2794" t="s">
         <v>2796</v>
@@ -48430,7 +48430,7 @@
         <v>14</v>
       </c>
       <c r="C2795">
-        <v>4900</v>
+        <v>5000</v>
       </c>
       <c r="D2795" t="s">
         <v>2797</v>
@@ -48444,7 +48444,7 @@
         <v>15</v>
       </c>
       <c r="C2796">
-        <v>4900</v>
+        <v>5020</v>
       </c>
       <c r="D2796" t="s">
         <v>2798</v>
@@ -48458,7 +48458,7 @@
         <v>16</v>
       </c>
       <c r="C2797">
-        <v>4910</v>
+        <v>5060</v>
       </c>
       <c r="D2797" t="s">
         <v>2799</v>
@@ -48472,7 +48472,7 @@
         <v>17</v>
       </c>
       <c r="C2798">
-        <v>4920</v>
+        <v>5110</v>
       </c>
       <c r="D2798" t="s">
         <v>2800</v>
@@ -48486,7 +48486,7 @@
         <v>18</v>
       </c>
       <c r="C2799">
-        <v>4940</v>
+        <v>5130</v>
       </c>
       <c r="D2799" t="s">
         <v>2801</v>
@@ -48500,7 +48500,7 @@
         <v>19</v>
       </c>
       <c r="C2800">
-        <v>4980</v>
+        <v>5150</v>
       </c>
       <c r="D2800" t="s">
         <v>2802</v>
@@ -48514,7 +48514,7 @@
         <v>20</v>
       </c>
       <c r="C2801">
-        <v>5020</v>
+        <v>5190</v>
       </c>
       <c r="D2801" t="s">
         <v>2803</v>
@@ -48528,7 +48528,7 @@
         <v>21</v>
       </c>
       <c r="C2802">
-        <v>5080</v>
+        <v>5230</v>
       </c>
       <c r="D2802" t="s">
         <v>2804</v>
@@ -48542,7 +48542,7 @@
         <v>22</v>
       </c>
       <c r="C2803">
-        <v>5160</v>
+        <v>5300</v>
       </c>
       <c r="D2803" t="s">
         <v>2805</v>
@@ -48556,7 +48556,7 @@
         <v>23</v>
       </c>
       <c r="C2804">
-        <v>5270</v>
+        <v>5390</v>
       </c>
       <c r="D2804" t="s">
         <v>2806</v>
@@ -48570,7 +48570,7 @@
         <v>24</v>
       </c>
       <c r="C2805">
-        <v>5400</v>
+        <v>5510</v>
       </c>
       <c r="D2805" t="s">
         <v>2807</v>
@@ -48584,7 +48584,7 @@
         <v>25</v>
       </c>
       <c r="C2806">
-        <v>5550</v>
+        <v>5650</v>
       </c>
       <c r="D2806" t="s">
         <v>2808</v>
@@ -48598,7 +48598,7 @@
         <v>26</v>
       </c>
       <c r="C2807">
-        <v>5710</v>
+        <v>5820</v>
       </c>
       <c r="D2807" t="s">
         <v>2809</v>
@@ -48612,7 +48612,7 @@
         <v>27</v>
       </c>
       <c r="C2808">
-        <v>5890</v>
+        <v>6000</v>
       </c>
       <c r="D2808" t="s">
         <v>2810</v>
@@ -48626,7 +48626,7 @@
         <v>28</v>
       </c>
       <c r="C2809">
-        <v>6080</v>
+        <v>6150</v>
       </c>
       <c r="D2809" t="s">
         <v>2811</v>
@@ -48640,7 +48640,7 @@
         <v>29</v>
       </c>
       <c r="C2810">
-        <v>6280</v>
+        <v>6330</v>
       </c>
       <c r="D2810" t="s">
         <v>2812</v>
@@ -48654,7 +48654,7 @@
         <v>30</v>
       </c>
       <c r="C2811">
-        <v>6470</v>
+        <v>6550</v>
       </c>
       <c r="D2811" t="s">
         <v>2813</v>
@@ -48668,7 +48668,7 @@
         <v>31</v>
       </c>
       <c r="C2812">
-        <v>6640</v>
+        <v>6700</v>
       </c>
       <c r="D2812" t="s">
         <v>2814</v>
@@ -48696,7 +48696,7 @@
         <v>33</v>
       </c>
       <c r="C2814">
-        <v>6940</v>
+        <v>6900</v>
       </c>
       <c r="D2814" t="s">
         <v>2816</v>
@@ -48710,7 +48710,7 @@
         <v>34</v>
       </c>
       <c r="C2815">
-        <v>7040</v>
+        <v>6950</v>
       </c>
       <c r="D2815" t="s">
         <v>2817</v>
@@ -48724,7 +48724,7 @@
         <v>35</v>
       </c>
       <c r="C2816">
-        <v>7100</v>
+        <v>6990</v>
       </c>
       <c r="D2816" t="s">
         <v>2818</v>
@@ -48738,7 +48738,7 @@
         <v>36</v>
       </c>
       <c r="C2817">
-        <v>7110</v>
+        <v>7000</v>
       </c>
       <c r="D2817" t="s">
         <v>2819</v>
@@ -48752,7 +48752,7 @@
         <v>37</v>
       </c>
       <c r="C2818">
-        <v>7090</v>
+        <v>7000</v>
       </c>
       <c r="D2818" t="s">
         <v>2820</v>
@@ -48766,7 +48766,7 @@
         <v>38</v>
       </c>
       <c r="C2819">
-        <v>7060</v>
+        <v>7000</v>
       </c>
       <c r="D2819" t="s">
         <v>2821</v>
@@ -48780,7 +48780,7 @@
         <v>39</v>
       </c>
       <c r="C2820">
-        <v>7020</v>
+        <v>7000</v>
       </c>
       <c r="D2820" t="s">
         <v>2822</v>
@@ -48794,7 +48794,7 @@
         <v>40</v>
       </c>
       <c r="C2821">
-        <v>6970</v>
+        <v>7000</v>
       </c>
       <c r="D2821" t="s">
         <v>2823</v>
@@ -48808,7 +48808,7 @@
         <v>41</v>
       </c>
       <c r="C2822">
-        <v>6910</v>
+        <v>6950</v>
       </c>
       <c r="D2822" t="s">
         <v>2824</v>
@@ -48822,7 +48822,7 @@
         <v>42</v>
       </c>
       <c r="C2823">
-        <v>6840</v>
+        <v>6920</v>
       </c>
       <c r="D2823" t="s">
         <v>2825</v>
@@ -48836,7 +48836,7 @@
         <v>43</v>
       </c>
       <c r="C2824">
-        <v>6760</v>
+        <v>6900</v>
       </c>
       <c r="D2824" t="s">
         <v>2826</v>
@@ -48850,7 +48850,7 @@
         <v>44</v>
       </c>
       <c r="C2825">
-        <v>6670</v>
+        <v>6840</v>
       </c>
       <c r="D2825" t="s">
         <v>2827</v>
@@ -48864,7 +48864,7 @@
         <v>45</v>
       </c>
       <c r="C2826">
-        <v>6570</v>
+        <v>6820</v>
       </c>
       <c r="D2826" t="s">
         <v>2828</v>
@@ -48878,7 +48878,7 @@
         <v>46</v>
       </c>
       <c r="C2827">
-        <v>6480</v>
+        <v>6770</v>
       </c>
       <c r="D2827" t="s">
         <v>2829</v>
@@ -48892,7 +48892,7 @@
         <v>47</v>
       </c>
       <c r="C2828">
-        <v>6390</v>
+        <v>6690</v>
       </c>
       <c r="D2828" t="s">
         <v>2830</v>
@@ -48906,7 +48906,7 @@
         <v>48</v>
       </c>
       <c r="C2829">
-        <v>6320</v>
+        <v>6610</v>
       </c>
       <c r="D2829" t="s">
         <v>2831</v>
@@ -48920,7 +48920,7 @@
         <v>49</v>
       </c>
       <c r="C2830">
-        <v>6260</v>
+        <v>6530</v>
       </c>
       <c r="D2830" t="s">
         <v>2832</v>
@@ -48934,7 +48934,7 @@
         <v>50</v>
       </c>
       <c r="C2831">
-        <v>6210</v>
+        <v>6470</v>
       </c>
       <c r="D2831" t="s">
         <v>2833</v>
@@ -48948,7 +48948,7 @@
         <v>51</v>
       </c>
       <c r="C2832">
-        <v>6180</v>
+        <v>6430</v>
       </c>
       <c r="D2832" t="s">
         <v>2834</v>
@@ -48962,7 +48962,7 @@
         <v>52</v>
       </c>
       <c r="C2833">
-        <v>6170</v>
+        <v>6410</v>
       </c>
       <c r="D2833" t="s">
         <v>2835</v>
@@ -48976,7 +48976,7 @@
         <v>53</v>
       </c>
       <c r="C2834">
-        <v>6170</v>
+        <v>6410</v>
       </c>
       <c r="D2834" t="s">
         <v>2836</v>
@@ -48990,7 +48990,7 @@
         <v>54</v>
       </c>
       <c r="C2835">
-        <v>6160</v>
+        <v>6390</v>
       </c>
       <c r="D2835" t="s">
         <v>2837</v>
@@ -49004,7 +49004,7 @@
         <v>55</v>
       </c>
       <c r="C2836">
-        <v>6130</v>
+        <v>6370</v>
       </c>
       <c r="D2836" t="s">
         <v>2838</v>
@@ -49018,7 +49018,7 @@
         <v>56</v>
       </c>
       <c r="C2837">
-        <v>6080</v>
+        <v>6340</v>
       </c>
       <c r="D2837" t="s">
         <v>2839</v>
@@ -49032,7 +49032,7 @@
         <v>57</v>
       </c>
       <c r="C2838">
-        <v>6030</v>
+        <v>6310</v>
       </c>
       <c r="D2838" t="s">
         <v>2840</v>
@@ -49046,7 +49046,7 @@
         <v>58</v>
       </c>
       <c r="C2839">
-        <v>6000</v>
+        <v>6280</v>
       </c>
       <c r="D2839" t="s">
         <v>2841</v>
@@ -49060,7 +49060,7 @@
         <v>59</v>
       </c>
       <c r="C2840">
-        <v>6010</v>
+        <v>6280</v>
       </c>
       <c r="D2840" t="s">
         <v>2842</v>
@@ -49074,7 +49074,7 @@
         <v>60</v>
       </c>
       <c r="C2841">
-        <v>6070</v>
+        <v>6300</v>
       </c>
       <c r="D2841" t="s">
         <v>2843</v>
@@ -49088,7 +49088,7 @@
         <v>61</v>
       </c>
       <c r="C2842">
-        <v>6150</v>
+        <v>6330</v>
       </c>
       <c r="D2842" t="s">
         <v>2844</v>
@@ -49102,7 +49102,7 @@
         <v>62</v>
       </c>
       <c r="C2843">
-        <v>6230</v>
+        <v>6360</v>
       </c>
       <c r="D2843" t="s">
         <v>2845</v>
@@ -49116,7 +49116,7 @@
         <v>63</v>
       </c>
       <c r="C2844">
-        <v>6280</v>
+        <v>6390</v>
       </c>
       <c r="D2844" t="s">
         <v>2846</v>
@@ -49130,7 +49130,7 @@
         <v>64</v>
       </c>
       <c r="C2845">
-        <v>6310</v>
+        <v>6420</v>
       </c>
       <c r="D2845" t="s">
         <v>2847</v>
@@ -49144,7 +49144,7 @@
         <v>65</v>
       </c>
       <c r="C2846">
-        <v>6320</v>
+        <v>6440</v>
       </c>
       <c r="D2846" t="s">
         <v>2848</v>
@@ -49158,7 +49158,7 @@
         <v>66</v>
       </c>
       <c r="C2847">
-        <v>6350</v>
+        <v>6480</v>
       </c>
       <c r="D2847" t="s">
         <v>2849</v>
@@ -49172,7 +49172,7 @@
         <v>67</v>
       </c>
       <c r="C2848">
-        <v>6400</v>
+        <v>6530</v>
       </c>
       <c r="D2848" t="s">
         <v>2850</v>
@@ -49186,7 +49186,7 @@
         <v>68</v>
       </c>
       <c r="C2849">
-        <v>6460</v>
+        <v>6600</v>
       </c>
       <c r="D2849" t="s">
         <v>2851</v>
@@ -49200,7 +49200,7 @@
         <v>69</v>
       </c>
       <c r="C2850">
-        <v>6530</v>
+        <v>6680</v>
       </c>
       <c r="D2850" t="s">
         <v>2852</v>
@@ -49214,7 +49214,7 @@
         <v>70</v>
       </c>
       <c r="C2851">
-        <v>6610</v>
+        <v>6760</v>
       </c>
       <c r="D2851" t="s">
         <v>2853</v>
@@ -49228,7 +49228,7 @@
         <v>71</v>
       </c>
       <c r="C2852">
-        <v>6680</v>
+        <v>6840</v>
       </c>
       <c r="D2852" t="s">
         <v>2854</v>
@@ -49242,7 +49242,7 @@
         <v>72</v>
       </c>
       <c r="C2853">
-        <v>6750</v>
+        <v>6910</v>
       </c>
       <c r="D2853" t="s">
         <v>2855</v>
@@ -49256,7 +49256,7 @@
         <v>73</v>
       </c>
       <c r="C2854">
-        <v>6810</v>
+        <v>6990</v>
       </c>
       <c r="D2854" t="s">
         <v>2856</v>
@@ -49270,7 +49270,7 @@
         <v>74</v>
       </c>
       <c r="C2855">
-        <v>6880</v>
+        <v>7060</v>
       </c>
       <c r="D2855" t="s">
         <v>2857</v>
@@ -49284,7 +49284,7 @@
         <v>75</v>
       </c>
       <c r="C2856">
-        <v>6940</v>
+        <v>7130</v>
       </c>
       <c r="D2856" t="s">
         <v>2858</v>
@@ -49298,7 +49298,7 @@
         <v>76</v>
       </c>
       <c r="C2857">
-        <v>7010</v>
+        <v>7200</v>
       </c>
       <c r="D2857" t="s">
         <v>2859</v>
@@ -49312,7 +49312,7 @@
         <v>77</v>
       </c>
       <c r="C2858">
-        <v>7070</v>
+        <v>7260</v>
       </c>
       <c r="D2858" t="s">
         <v>2860</v>
@@ -49326,7 +49326,7 @@
         <v>78</v>
       </c>
       <c r="C2859">
-        <v>7150</v>
+        <v>7340</v>
       </c>
       <c r="D2859" t="s">
         <v>2861</v>
@@ -49340,7 +49340,7 @@
         <v>79</v>
       </c>
       <c r="C2860">
-        <v>7240</v>
+        <v>7430</v>
       </c>
       <c r="D2860" t="s">
         <v>2862</v>
@@ -49354,7 +49354,7 @@
         <v>80</v>
       </c>
       <c r="C2861">
-        <v>7350</v>
+        <v>7530</v>
       </c>
       <c r="D2861" t="s">
         <v>2863</v>
@@ -49368,7 +49368,7 @@
         <v>81</v>
       </c>
       <c r="C2862">
-        <v>7460</v>
+        <v>7600</v>
       </c>
       <c r="D2862" t="s">
         <v>2864</v>
@@ -49382,7 +49382,7 @@
         <v>82</v>
       </c>
       <c r="C2863">
-        <v>7530</v>
+        <v>7620</v>
       </c>
       <c r="D2863" t="s">
         <v>2865</v>
@@ -49396,7 +49396,7 @@
         <v>83</v>
       </c>
       <c r="C2864">
-        <v>7540</v>
+        <v>7650</v>
       </c>
       <c r="D2864" t="s">
         <v>2866</v>
@@ -49410,7 +49410,7 @@
         <v>84</v>
       </c>
       <c r="C2865">
-        <v>7500</v>
+        <v>7650</v>
       </c>
       <c r="D2865" t="s">
         <v>2867</v>
@@ -49424,7 +49424,7 @@
         <v>85</v>
       </c>
       <c r="C2866">
-        <v>7400</v>
+        <v>7600</v>
       </c>
       <c r="D2866" t="s">
         <v>2868</v>
@@ -49438,7 +49438,7 @@
         <v>86</v>
       </c>
       <c r="C2867">
-        <v>7290</v>
+        <v>7430</v>
       </c>
       <c r="D2867" t="s">
         <v>2869</v>
@@ -49452,7 +49452,7 @@
         <v>87</v>
       </c>
       <c r="C2868">
-        <v>7150</v>
+        <v>7300</v>
       </c>
       <c r="D2868" t="s">
         <v>2870</v>
@@ -49466,7 +49466,7 @@
         <v>88</v>
       </c>
       <c r="C2869">
-        <v>7000</v>
+        <v>7160</v>
       </c>
       <c r="D2869" t="s">
         <v>2871</v>
@@ -49480,7 +49480,7 @@
         <v>89</v>
       </c>
       <c r="C2870">
-        <v>6840</v>
+        <v>7000</v>
       </c>
       <c r="D2870" t="s">
         <v>2872</v>
@@ -49494,7 +49494,7 @@
         <v>90</v>
       </c>
       <c r="C2871">
-        <v>6680</v>
+        <v>6840</v>
       </c>
       <c r="D2871" t="s">
         <v>2873</v>
@@ -49508,7 +49508,7 @@
         <v>91</v>
       </c>
       <c r="C2872">
-        <v>6520</v>
+        <v>6690</v>
       </c>
       <c r="D2872" t="s">
         <v>2874</v>
@@ -49522,7 +49522,7 @@
         <v>92</v>
       </c>
       <c r="C2873">
-        <v>6370</v>
+        <v>6530</v>
       </c>
       <c r="D2873" t="s">
         <v>2875</v>
@@ -49536,7 +49536,7 @@
         <v>93</v>
       </c>
       <c r="C2874">
-        <v>6230</v>
+        <v>6370</v>
       </c>
       <c r="D2874" t="s">
         <v>2876</v>
@@ -49550,7 +49550,7 @@
         <v>94</v>
       </c>
       <c r="C2875">
-        <v>6100</v>
+        <v>6240</v>
       </c>
       <c r="D2875" t="s">
         <v>2877</v>
@@ -49564,7 +49564,7 @@
         <v>95</v>
       </c>
       <c r="C2876">
-        <v>5980</v>
+        <v>6120</v>
       </c>
       <c r="D2876" t="s">
         <v>2878</v>
@@ -49578,7 +49578,7 @@
         <v>96</v>
       </c>
       <c r="C2877">
-        <v>5880</v>
+        <v>6030</v>
       </c>
       <c r="D2877" t="s">
         <v>2879</v>
@@ -49592,7 +49592,7 @@
         <v>1</v>
       </c>
       <c r="C2878">
-        <v>5800</v>
+        <v>5950</v>
       </c>
       <c r="D2878" t="s">
         <v>2880</v>
@@ -49606,7 +49606,7 @@
         <v>2</v>
       </c>
       <c r="C2879">
-        <v>5730</v>
+        <v>5880</v>
       </c>
       <c r="D2879" t="s">
         <v>2881</v>
@@ -49620,7 +49620,7 @@
         <v>3</v>
       </c>
       <c r="C2880">
-        <v>5670</v>
+        <v>5820</v>
       </c>
       <c r="D2880" t="s">
         <v>2882</v>
@@ -49634,7 +49634,7 @@
         <v>4</v>
       </c>
       <c r="C2881">
-        <v>5620</v>
+        <v>5760</v>
       </c>
       <c r="D2881" t="s">
         <v>2883</v>
@@ -49648,7 +49648,7 @@
         <v>5</v>
       </c>
       <c r="C2882">
-        <v>5580</v>
+        <v>5710</v>
       </c>
       <c r="D2882" t="s">
         <v>2884</v>
@@ -49662,7 +49662,7 @@
         <v>6</v>
       </c>
       <c r="C2883">
-        <v>5550</v>
+        <v>5670</v>
       </c>
       <c r="D2883" t="s">
         <v>2885</v>
@@ -49676,7 +49676,7 @@
         <v>7</v>
       </c>
       <c r="C2884">
-        <v>5510</v>
+        <v>5630</v>
       </c>
       <c r="D2884" t="s">
         <v>2886</v>
@@ -49690,7 +49690,7 @@
         <v>8</v>
       </c>
       <c r="C2885">
-        <v>5480</v>
+        <v>5600</v>
       </c>
       <c r="D2885" t="s">
         <v>2887</v>
@@ -49704,7 +49704,7 @@
         <v>9</v>
       </c>
       <c r="C2886">
-        <v>5450</v>
+        <v>5580</v>
       </c>
       <c r="D2886" t="s">
         <v>2888</v>
@@ -49718,7 +49718,7 @@
         <v>10</v>
       </c>
       <c r="C2887">
-        <v>5430</v>
+        <v>5560</v>
       </c>
       <c r="D2887" t="s">
         <v>2889</v>
@@ -49732,7 +49732,7 @@
         <v>11</v>
       </c>
       <c r="C2888">
-        <v>5410</v>
+        <v>5550</v>
       </c>
       <c r="D2888" t="s">
         <v>2890</v>
@@ -49746,7 +49746,7 @@
         <v>12</v>
       </c>
       <c r="C2889">
-        <v>5400</v>
+        <v>5540</v>
       </c>
       <c r="D2889" t="s">
         <v>2891</v>
@@ -49760,7 +49760,7 @@
         <v>13</v>
       </c>
       <c r="C2890">
-        <v>5400</v>
+        <v>5520</v>
       </c>
       <c r="D2890" t="s">
         <v>2892</v>
@@ -49774,7 +49774,7 @@
         <v>14</v>
       </c>
       <c r="C2891">
-        <v>5400</v>
+        <v>5500</v>
       </c>
       <c r="D2891" t="s">
         <v>2893</v>
@@ -49788,7 +49788,7 @@
         <v>15</v>
       </c>
       <c r="C2892">
-        <v>5410</v>
+        <v>5520</v>
       </c>
       <c r="D2892" t="s">
         <v>2894</v>
@@ -49802,7 +49802,7 @@
         <v>16</v>
       </c>
       <c r="C2893">
-        <v>5420</v>
+        <v>5530</v>
       </c>
       <c r="D2893" t="s">
         <v>2895</v>
@@ -49816,7 +49816,7 @@
         <v>17</v>
       </c>
       <c r="C2894">
-        <v>5440</v>
+        <v>5550</v>
       </c>
       <c r="D2894" t="s">
         <v>2896</v>
@@ -49830,7 +49830,7 @@
         <v>18</v>
       </c>
       <c r="C2895">
-        <v>5460</v>
+        <v>5590</v>
       </c>
       <c r="D2895" t="s">
         <v>2897</v>
@@ -49844,7 +49844,7 @@
         <v>19</v>
       </c>
       <c r="C2896">
-        <v>5490</v>
+        <v>5620</v>
       </c>
       <c r="D2896" t="s">
         <v>2898</v>
@@ -49858,7 +49858,7 @@
         <v>20</v>
       </c>
       <c r="C2897">
-        <v>5520</v>
+        <v>5650</v>
       </c>
       <c r="D2897" t="s">
         <v>2899</v>
@@ -49872,7 +49872,7 @@
         <v>21</v>
       </c>
       <c r="C2898">
-        <v>5560</v>
+        <v>5690</v>
       </c>
       <c r="D2898" t="s">
         <v>2900</v>
@@ -49886,7 +49886,7 @@
         <v>22</v>
       </c>
       <c r="C2899">
-        <v>5610</v>
+        <v>5750</v>
       </c>
       <c r="D2899" t="s">
         <v>2901</v>
@@ -49900,7 +49900,7 @@
         <v>23</v>
       </c>
       <c r="C2900">
-        <v>5690</v>
+        <v>5820</v>
       </c>
       <c r="D2900" t="s">
         <v>2902</v>
@@ -49914,7 +49914,7 @@
         <v>24</v>
       </c>
       <c r="C2901">
-        <v>5790</v>
+        <v>5900</v>
       </c>
       <c r="D2901" t="s">
         <v>2903</v>
@@ -49928,7 +49928,7 @@
         <v>25</v>
       </c>
       <c r="C2902">
-        <v>5900</v>
+        <v>5990</v>
       </c>
       <c r="D2902" t="s">
         <v>2904</v>
@@ -49942,7 +49942,7 @@
         <v>26</v>
       </c>
       <c r="C2903">
-        <v>6030</v>
+        <v>6110</v>
       </c>
       <c r="D2903" t="s">
         <v>2905</v>
@@ -49956,7 +49956,7 @@
         <v>27</v>
       </c>
       <c r="C2904">
-        <v>6190</v>
+        <v>6260</v>
       </c>
       <c r="D2904" t="s">
         <v>2906</v>
@@ -49970,7 +49970,7 @@
         <v>28</v>
       </c>
       <c r="C2905">
-        <v>6360</v>
+        <v>6430</v>
       </c>
       <c r="D2905" t="s">
         <v>2907</v>
@@ -49984,7 +49984,7 @@
         <v>29</v>
       </c>
       <c r="C2906">
-        <v>6540</v>
+        <v>6620</v>
       </c>
       <c r="D2906" t="s">
         <v>2908</v>
@@ -49998,7 +49998,7 @@
         <v>30</v>
       </c>
       <c r="C2907">
-        <v>6710</v>
+        <v>6750</v>
       </c>
       <c r="D2907" t="s">
         <v>2909</v>
@@ -50012,7 +50012,7 @@
         <v>31</v>
       </c>
       <c r="C2908">
-        <v>6850</v>
+        <v>6780</v>
       </c>
       <c r="D2908" t="s">
         <v>2910</v>
@@ -50026,7 +50026,7 @@
         <v>32</v>
       </c>
       <c r="C2909">
-        <v>6980</v>
+        <v>6850</v>
       </c>
       <c r="D2909" t="s">
         <v>2911</v>
@@ -50040,7 +50040,7 @@
         <v>33</v>
       </c>
       <c r="C2910">
-        <v>7080</v>
+        <v>6950</v>
       </c>
       <c r="D2910" t="s">
         <v>2912</v>
@@ -50054,7 +50054,7 @@
         <v>34</v>
       </c>
       <c r="C2911">
-        <v>7150</v>
+        <v>7000</v>
       </c>
       <c r="D2911" t="s">
         <v>2913</v>
@@ -50068,7 +50068,7 @@
         <v>35</v>
       </c>
       <c r="C2912">
-        <v>7200</v>
+        <v>7060</v>
       </c>
       <c r="D2912" t="s">
         <v>2914</v>
@@ -50082,7 +50082,7 @@
         <v>36</v>
       </c>
       <c r="C2913">
-        <v>7200</v>
+        <v>7080</v>
       </c>
       <c r="D2913" t="s">
         <v>2915</v>
@@ -50096,7 +50096,7 @@
         <v>37</v>
       </c>
       <c r="C2914">
-        <v>7190</v>
+        <v>7100</v>
       </c>
       <c r="D2914" t="s">
         <v>2916</v>
@@ -50110,7 +50110,7 @@
         <v>38</v>
       </c>
       <c r="C2915">
-        <v>7150</v>
+        <v>7100</v>
       </c>
       <c r="D2915" t="s">
         <v>2917</v>
@@ -50124,7 +50124,7 @@
         <v>39</v>
       </c>
       <c r="C2916">
-        <v>7110</v>
+        <v>7100</v>
       </c>
       <c r="D2916" t="s">
         <v>2918</v>
@@ -50138,7 +50138,7 @@
         <v>40</v>
       </c>
       <c r="C2917">
-        <v>7050</v>
+        <v>7080</v>
       </c>
       <c r="D2917" t="s">
         <v>2919</v>
@@ -50152,7 +50152,7 @@
         <v>41</v>
       </c>
       <c r="C2918">
-        <v>6980</v>
+        <v>7020</v>
       </c>
       <c r="D2918" t="s">
         <v>2920</v>
@@ -50166,7 +50166,7 @@
         <v>42</v>
       </c>
       <c r="C2919">
-        <v>6900</v>
+        <v>6930</v>
       </c>
       <c r="D2919" t="s">
         <v>2921</v>
@@ -50180,7 +50180,7 @@
         <v>43</v>
       </c>
       <c r="C2920">
-        <v>6820</v>
+        <v>6850</v>
       </c>
       <c r="D2920" t="s">
         <v>2922</v>
@@ -50194,7 +50194,7 @@
         <v>44</v>
       </c>
       <c r="C2921">
-        <v>6720</v>
+        <v>6750</v>
       </c>
       <c r="D2921" t="s">
         <v>2923</v>
@@ -50208,7 +50208,7 @@
         <v>45</v>
       </c>
       <c r="C2922">
-        <v>6610</v>
+        <v>6640</v>
       </c>
       <c r="D2922" t="s">
         <v>2924</v>
@@ -50222,7 +50222,7 @@
         <v>46</v>
       </c>
       <c r="C2923">
-        <v>6520</v>
+        <v>6540</v>
       </c>
       <c r="D2923" t="s">
         <v>2925</v>
@@ -50236,7 +50236,7 @@
         <v>47</v>
       </c>
       <c r="C2924">
-        <v>6430</v>
+        <v>6460</v>
       </c>
       <c r="D2924" t="s">
         <v>2926</v>
@@ -50250,7 +50250,7 @@
         <v>48</v>
       </c>
       <c r="C2925">
-        <v>6360</v>
+        <v>6380</v>
       </c>
       <c r="D2925" t="s">
         <v>2927</v>
@@ -50264,7 +50264,7 @@
         <v>49</v>
       </c>
       <c r="C2926">
-        <v>6300</v>
+        <v>6320</v>
       </c>
       <c r="D2926" t="s">
         <v>2928</v>
@@ -50278,7 +50278,7 @@
         <v>50</v>
       </c>
       <c r="C2927">
-        <v>6250</v>
+        <v>6270</v>
       </c>
       <c r="D2927" t="s">
         <v>2929</v>
@@ -50292,7 +50292,7 @@
         <v>51</v>
       </c>
       <c r="C2928">
-        <v>6220</v>
+        <v>6240</v>
       </c>
       <c r="D2928" t="s">
         <v>2930</v>
@@ -50306,7 +50306,7 @@
         <v>52</v>
       </c>
       <c r="C2929">
-        <v>6200</v>
+        <v>6230</v>
       </c>
       <c r="D2929" t="s">
         <v>2931</v>
@@ -50320,7 +50320,7 @@
         <v>53</v>
       </c>
       <c r="C2930">
-        <v>6200</v>
+        <v>6220</v>
       </c>
       <c r="D2930" t="s">
         <v>2932</v>
@@ -50334,7 +50334,7 @@
         <v>54</v>
       </c>
       <c r="C2931">
-        <v>6180</v>
+        <v>6210</v>
       </c>
       <c r="D2931" t="s">
         <v>2933</v>
@@ -50348,7 +50348,7 @@
         <v>55</v>
       </c>
       <c r="C2932">
-        <v>6160</v>
+        <v>6190</v>
       </c>
       <c r="D2932" t="s">
         <v>2934</v>
@@ -50362,7 +50362,7 @@
         <v>56</v>
       </c>
       <c r="C2933">
-        <v>6120</v>
+        <v>6160</v>
       </c>
       <c r="D2933" t="s">
         <v>2935</v>
@@ -50376,7 +50376,7 @@
         <v>57</v>
       </c>
       <c r="C2934">
-        <v>6080</v>
+        <v>6130</v>
       </c>
       <c r="D2934" t="s">
         <v>2936</v>
@@ -50390,7 +50390,7 @@
         <v>58</v>
       </c>
       <c r="C2935">
-        <v>6050</v>
+        <v>6110</v>
       </c>
       <c r="D2935" t="s">
         <v>2937</v>
@@ -50404,7 +50404,7 @@
         <v>59</v>
       </c>
       <c r="C2936">
-        <v>6050</v>
+        <v>6100</v>
       </c>
       <c r="D2936" t="s">
         <v>2938</v>
@@ -50418,7 +50418,7 @@
         <v>60</v>
       </c>
       <c r="C2937">
-        <v>6080</v>
+        <v>6110</v>
       </c>
       <c r="D2937" t="s">
         <v>2939</v>
@@ -50446,7 +50446,7 @@
         <v>62</v>
       </c>
       <c r="C2939">
-        <v>6170</v>
+        <v>6160</v>
       </c>
       <c r="D2939" t="s">
         <v>2941</v>
@@ -50460,7 +50460,7 @@
         <v>63</v>
       </c>
       <c r="C2940">
-        <v>6210</v>
+        <v>6190</v>
       </c>
       <c r="D2940" t="s">
         <v>2942</v>
@@ -50474,7 +50474,7 @@
         <v>64</v>
       </c>
       <c r="C2941">
-        <v>6250</v>
+        <v>6230</v>
       </c>
       <c r="D2941" t="s">
         <v>2943</v>
@@ -50488,7 +50488,7 @@
         <v>65</v>
       </c>
       <c r="C2942">
-        <v>6270</v>
+        <v>6280</v>
       </c>
       <c r="D2942" t="s">
         <v>2944</v>
@@ -50502,7 +50502,7 @@
         <v>66</v>
       </c>
       <c r="C2943">
-        <v>6310</v>
+        <v>6330</v>
       </c>
       <c r="D2943" t="s">
         <v>2945</v>
@@ -50516,7 +50516,7 @@
         <v>67</v>
       </c>
       <c r="C2944">
-        <v>6360</v>
+        <v>6400</v>
       </c>
       <c r="D2944" t="s">
         <v>2946</v>
@@ -50530,7 +50530,7 @@
         <v>68</v>
       </c>
       <c r="C2945">
-        <v>6420</v>
+        <v>6480</v>
       </c>
       <c r="D2945" t="s">
         <v>2947</v>
@@ -50544,7 +50544,7 @@
         <v>69</v>
       </c>
       <c r="C2946">
-        <v>6500</v>
+        <v>6580</v>
       </c>
       <c r="D2946" t="s">
         <v>2948</v>
@@ -50558,7 +50558,7 @@
         <v>70</v>
       </c>
       <c r="C2947">
-        <v>6570</v>
+        <v>6670</v>
       </c>
       <c r="D2947" t="s">
         <v>2949</v>
@@ -50572,7 +50572,7 @@
         <v>71</v>
       </c>
       <c r="C2948">
-        <v>6650</v>
+        <v>6760</v>
       </c>
       <c r="D2948" t="s">
         <v>2950</v>
@@ -50586,7 +50586,7 @@
         <v>72</v>
       </c>
       <c r="C2949">
-        <v>6720</v>
+        <v>6860</v>
       </c>
       <c r="D2949" t="s">
         <v>2951</v>
@@ -50600,7 +50600,7 @@
         <v>73</v>
       </c>
       <c r="C2950">
-        <v>6800</v>
+        <v>6950</v>
       </c>
       <c r="D2950" t="s">
         <v>2952</v>
@@ -50614,7 +50614,7 @@
         <v>74</v>
       </c>
       <c r="C2951">
-        <v>6870</v>
+        <v>7030</v>
       </c>
       <c r="D2951" t="s">
         <v>2953</v>
@@ -50628,7 +50628,7 @@
         <v>75</v>
       </c>
       <c r="C2952">
-        <v>6940</v>
+        <v>7110</v>
       </c>
       <c r="D2952" t="s">
         <v>2954</v>
@@ -50642,7 +50642,7 @@
         <v>76</v>
       </c>
       <c r="C2953">
-        <v>7010</v>
+        <v>7180</v>
       </c>
       <c r="D2953" t="s">
         <v>2955</v>
@@ -50656,7 +50656,7 @@
         <v>77</v>
       </c>
       <c r="C2954">
-        <v>7080</v>
+        <v>7250</v>
       </c>
       <c r="D2954" t="s">
         <v>2956</v>
@@ -50670,7 +50670,7 @@
         <v>78</v>
       </c>
       <c r="C2955">
-        <v>7150</v>
+        <v>7330</v>
       </c>
       <c r="D2955" t="s">
         <v>2957</v>
@@ -50684,7 +50684,7 @@
         <v>79</v>
       </c>
       <c r="C2956">
-        <v>7250</v>
+        <v>7440</v>
       </c>
       <c r="D2956" t="s">
         <v>2958</v>
@@ -50698,7 +50698,7 @@
         <v>80</v>
       </c>
       <c r="C2957">
-        <v>7360</v>
+        <v>7550</v>
       </c>
       <c r="D2957" t="s">
         <v>2959</v>
@@ -50712,7 +50712,7 @@
         <v>81</v>
       </c>
       <c r="C2958">
-        <v>7480</v>
+        <v>7580</v>
       </c>
       <c r="D2958" t="s">
         <v>2960</v>
@@ -50726,7 +50726,7 @@
         <v>82</v>
       </c>
       <c r="C2959">
-        <v>7550</v>
+        <v>7650</v>
       </c>
       <c r="D2959" t="s">
         <v>2961</v>
@@ -50740,7 +50740,7 @@
         <v>83</v>
       </c>
       <c r="C2960">
-        <v>7560</v>
+        <v>7700</v>
       </c>
       <c r="D2960" t="s">
         <v>2962</v>
@@ -50754,7 +50754,7 @@
         <v>84</v>
       </c>
       <c r="C2961">
-        <v>7520</v>
+        <v>7700</v>
       </c>
       <c r="D2961" t="s">
         <v>2963</v>
@@ -50768,7 +50768,7 @@
         <v>85</v>
       </c>
       <c r="C2962">
-        <v>7430</v>
+        <v>7620</v>
       </c>
       <c r="D2962" t="s">
         <v>2964</v>
@@ -50782,7 +50782,7 @@
         <v>86</v>
       </c>
       <c r="C2963">
-        <v>7310</v>
+        <v>7500</v>
       </c>
       <c r="D2963" t="s">
         <v>2965</v>
@@ -50796,7 +50796,7 @@
         <v>87</v>
       </c>
       <c r="C2964">
-        <v>7180</v>
+        <v>7370</v>
       </c>
       <c r="D2964" t="s">
         <v>2966</v>
@@ -50810,7 +50810,7 @@
         <v>88</v>
       </c>
       <c r="C2965">
-        <v>7030</v>
+        <v>7220</v>
       </c>
       <c r="D2965" t="s">
         <v>2967</v>
@@ -50824,7 +50824,7 @@
         <v>89</v>
       </c>
       <c r="C2966">
-        <v>6870</v>
+        <v>7070</v>
       </c>
       <c r="D2966" t="s">
         <v>2968</v>
@@ -50838,7 +50838,7 @@
         <v>90</v>
       </c>
       <c r="C2967">
-        <v>6710</v>
+        <v>6910</v>
       </c>
       <c r="D2967" t="s">
         <v>2969</v>
@@ -50852,7 +50852,7 @@
         <v>91</v>
       </c>
       <c r="C2968">
-        <v>6560</v>
+        <v>6760</v>
       </c>
       <c r="D2968" t="s">
         <v>2970</v>
@@ -50866,7 +50866,7 @@
         <v>92</v>
       </c>
       <c r="C2969">
-        <v>6410</v>
+        <v>6600</v>
       </c>
       <c r="D2969" t="s">
         <v>2971</v>
@@ -50880,7 +50880,7 @@
         <v>93</v>
       </c>
       <c r="C2970">
-        <v>6260</v>
+        <v>6450</v>
       </c>
       <c r="D2970" t="s">
         <v>2972</v>
@@ -50894,7 +50894,7 @@
         <v>94</v>
       </c>
       <c r="C2971">
-        <v>6130</v>
+        <v>6310</v>
       </c>
       <c r="D2971" t="s">
         <v>2973</v>
@@ -50908,7 +50908,7 @@
         <v>95</v>
       </c>
       <c r="C2972">
-        <v>6010</v>
+        <v>6190</v>
       </c>
       <c r="D2972" t="s">
         <v>2974</v>
@@ -50922,7 +50922,7 @@
         <v>96</v>
       </c>
       <c r="C2973">
-        <v>5910</v>
+        <v>6090</v>
       </c>
       <c r="D2973" t="s">
         <v>2975</v>

</xml_diff>

<commit_message>
Updating the Adrem model
</commit_message>
<xml_diff>
--- a/Market Fundamentals/Transelectrica_data/Cons_Prod_final/Weekly_Consumption_2026.xlsx
+++ b/Market Fundamentals/Transelectrica_data/Cons_Prod_final/Weekly_Consumption_2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1828" uniqueCount="1828">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1924" uniqueCount="1924">
   <si>
     <t>Date</t>
   </si>
@@ -5498,6 +5498,294 @@
   </si>
   <si>
     <t>19.05.202696.0</t>
+  </si>
+  <si>
+    <t>20.05.20261.0</t>
+  </si>
+  <si>
+    <t>20.05.20262.0</t>
+  </si>
+  <si>
+    <t>20.05.20263.0</t>
+  </si>
+  <si>
+    <t>20.05.20264.0</t>
+  </si>
+  <si>
+    <t>20.05.20265.0</t>
+  </si>
+  <si>
+    <t>20.05.20266.0</t>
+  </si>
+  <si>
+    <t>20.05.20267.0</t>
+  </si>
+  <si>
+    <t>20.05.20268.0</t>
+  </si>
+  <si>
+    <t>20.05.20269.0</t>
+  </si>
+  <si>
+    <t>20.05.202610.0</t>
+  </si>
+  <si>
+    <t>20.05.202611.0</t>
+  </si>
+  <si>
+    <t>20.05.202612.0</t>
+  </si>
+  <si>
+    <t>20.05.202613.0</t>
+  </si>
+  <si>
+    <t>20.05.202614.0</t>
+  </si>
+  <si>
+    <t>20.05.202615.0</t>
+  </si>
+  <si>
+    <t>20.05.202616.0</t>
+  </si>
+  <si>
+    <t>20.05.202617.0</t>
+  </si>
+  <si>
+    <t>20.05.202618.0</t>
+  </si>
+  <si>
+    <t>20.05.202619.0</t>
+  </si>
+  <si>
+    <t>20.05.202620.0</t>
+  </si>
+  <si>
+    <t>20.05.202621.0</t>
+  </si>
+  <si>
+    <t>20.05.202622.0</t>
+  </si>
+  <si>
+    <t>20.05.202623.0</t>
+  </si>
+  <si>
+    <t>20.05.202624.0</t>
+  </si>
+  <si>
+    <t>20.05.202625.0</t>
+  </si>
+  <si>
+    <t>20.05.202626.0</t>
+  </si>
+  <si>
+    <t>20.05.202627.0</t>
+  </si>
+  <si>
+    <t>20.05.202628.0</t>
+  </si>
+  <si>
+    <t>20.05.202629.0</t>
+  </si>
+  <si>
+    <t>20.05.202630.0</t>
+  </si>
+  <si>
+    <t>20.05.202631.0</t>
+  </si>
+  <si>
+    <t>20.05.202632.0</t>
+  </si>
+  <si>
+    <t>20.05.202633.0</t>
+  </si>
+  <si>
+    <t>20.05.202634.0</t>
+  </si>
+  <si>
+    <t>20.05.202635.0</t>
+  </si>
+  <si>
+    <t>20.05.202636.0</t>
+  </si>
+  <si>
+    <t>20.05.202637.0</t>
+  </si>
+  <si>
+    <t>20.05.202638.0</t>
+  </si>
+  <si>
+    <t>20.05.202639.0</t>
+  </si>
+  <si>
+    <t>20.05.202640.0</t>
+  </si>
+  <si>
+    <t>20.05.202641.0</t>
+  </si>
+  <si>
+    <t>20.05.202642.0</t>
+  </si>
+  <si>
+    <t>20.05.202643.0</t>
+  </si>
+  <si>
+    <t>20.05.202644.0</t>
+  </si>
+  <si>
+    <t>20.05.202645.0</t>
+  </si>
+  <si>
+    <t>20.05.202646.0</t>
+  </si>
+  <si>
+    <t>20.05.202647.0</t>
+  </si>
+  <si>
+    <t>20.05.202648.0</t>
+  </si>
+  <si>
+    <t>20.05.202649.0</t>
+  </si>
+  <si>
+    <t>20.05.202650.0</t>
+  </si>
+  <si>
+    <t>20.05.202651.0</t>
+  </si>
+  <si>
+    <t>20.05.202652.0</t>
+  </si>
+  <si>
+    <t>20.05.202653.0</t>
+  </si>
+  <si>
+    <t>20.05.202654.0</t>
+  </si>
+  <si>
+    <t>20.05.202655.0</t>
+  </si>
+  <si>
+    <t>20.05.202656.0</t>
+  </si>
+  <si>
+    <t>20.05.202657.0</t>
+  </si>
+  <si>
+    <t>20.05.202658.0</t>
+  </si>
+  <si>
+    <t>20.05.202659.0</t>
+  </si>
+  <si>
+    <t>20.05.202660.0</t>
+  </si>
+  <si>
+    <t>20.05.202661.0</t>
+  </si>
+  <si>
+    <t>20.05.202662.0</t>
+  </si>
+  <si>
+    <t>20.05.202663.0</t>
+  </si>
+  <si>
+    <t>20.05.202664.0</t>
+  </si>
+  <si>
+    <t>20.05.202665.0</t>
+  </si>
+  <si>
+    <t>20.05.202666.0</t>
+  </si>
+  <si>
+    <t>20.05.202667.0</t>
+  </si>
+  <si>
+    <t>20.05.202668.0</t>
+  </si>
+  <si>
+    <t>20.05.202669.0</t>
+  </si>
+  <si>
+    <t>20.05.202670.0</t>
+  </si>
+  <si>
+    <t>20.05.202671.0</t>
+  </si>
+  <si>
+    <t>20.05.202672.0</t>
+  </si>
+  <si>
+    <t>20.05.202673.0</t>
+  </si>
+  <si>
+    <t>20.05.202674.0</t>
+  </si>
+  <si>
+    <t>20.05.202675.0</t>
+  </si>
+  <si>
+    <t>20.05.202676.0</t>
+  </si>
+  <si>
+    <t>20.05.202677.0</t>
+  </si>
+  <si>
+    <t>20.05.202678.0</t>
+  </si>
+  <si>
+    <t>20.05.202679.0</t>
+  </si>
+  <si>
+    <t>20.05.202680.0</t>
+  </si>
+  <si>
+    <t>20.05.202681.0</t>
+  </si>
+  <si>
+    <t>20.05.202682.0</t>
+  </si>
+  <si>
+    <t>20.05.202683.0</t>
+  </si>
+  <si>
+    <t>20.05.202684.0</t>
+  </si>
+  <si>
+    <t>20.05.202685.0</t>
+  </si>
+  <si>
+    <t>20.05.202686.0</t>
+  </si>
+  <si>
+    <t>20.05.202687.0</t>
+  </si>
+  <si>
+    <t>20.05.202688.0</t>
+  </si>
+  <si>
+    <t>20.05.202689.0</t>
+  </si>
+  <si>
+    <t>20.05.202690.0</t>
+  </si>
+  <si>
+    <t>20.05.202691.0</t>
+  </si>
+  <si>
+    <t>20.05.202692.0</t>
+  </si>
+  <si>
+    <t>20.05.202693.0</t>
+  </si>
+  <si>
+    <t>20.05.202694.0</t>
+  </si>
+  <si>
+    <t>20.05.202695.0</t>
+  </si>
+  <si>
+    <t>20.05.202696.0</t>
   </si>
 </sst>
 </file>
@@ -5859,7 +6147,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D1825"/>
+  <dimension ref="A1:D1921"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:4">
@@ -22012,7 +22300,7 @@
         <v>1</v>
       </c>
       <c r="C1154">
-        <v>5500</v>
+        <v>5470</v>
       </c>
       <c r="D1154" t="s">
         <v>1156</v>
@@ -22026,7 +22314,7 @@
         <v>2</v>
       </c>
       <c r="C1155">
-        <v>5450</v>
+        <v>5410</v>
       </c>
       <c r="D1155" t="s">
         <v>1157</v>
@@ -22040,7 +22328,7 @@
         <v>3</v>
       </c>
       <c r="C1156">
-        <v>5390</v>
+        <v>5350</v>
       </c>
       <c r="D1156" t="s">
         <v>1158</v>
@@ -22054,7 +22342,7 @@
         <v>4</v>
       </c>
       <c r="C1157">
-        <v>5320</v>
+        <v>5300</v>
       </c>
       <c r="D1157" t="s">
         <v>1159</v>
@@ -22068,7 +22356,7 @@
         <v>5</v>
       </c>
       <c r="C1158">
-        <v>5260</v>
+        <v>5220</v>
       </c>
       <c r="D1158" t="s">
         <v>1160</v>
@@ -22082,7 +22370,7 @@
         <v>6</v>
       </c>
       <c r="C1159">
-        <v>5220</v>
+        <v>5190</v>
       </c>
       <c r="D1159" t="s">
         <v>1161</v>
@@ -22110,7 +22398,7 @@
         <v>8</v>
       </c>
       <c r="C1161">
-        <v>5130</v>
+        <v>5150</v>
       </c>
       <c r="D1161" t="s">
         <v>1163</v>
@@ -22124,7 +22412,7 @@
         <v>9</v>
       </c>
       <c r="C1162">
-        <v>5100</v>
+        <v>5090</v>
       </c>
       <c r="D1162" t="s">
         <v>1164</v>
@@ -22152,7 +22440,7 @@
         <v>11</v>
       </c>
       <c r="C1164">
-        <v>5070</v>
+        <v>5080</v>
       </c>
       <c r="D1164" t="s">
         <v>1166</v>
@@ -22166,7 +22454,7 @@
         <v>12</v>
       </c>
       <c r="C1165">
-        <v>5060</v>
+        <v>5080</v>
       </c>
       <c r="D1165" t="s">
         <v>1167</v>
@@ -22180,7 +22468,7 @@
         <v>13</v>
       </c>
       <c r="C1166">
-        <v>5050</v>
+        <v>5070</v>
       </c>
       <c r="D1166" t="s">
         <v>1168</v>
@@ -22194,7 +22482,7 @@
         <v>14</v>
       </c>
       <c r="C1167">
-        <v>5050</v>
+        <v>5070</v>
       </c>
       <c r="D1167" t="s">
         <v>1169</v>
@@ -22208,7 +22496,7 @@
         <v>15</v>
       </c>
       <c r="C1168">
-        <v>5050</v>
+        <v>5070</v>
       </c>
       <c r="D1168" t="s">
         <v>1170</v>
@@ -22222,7 +22510,7 @@
         <v>16</v>
       </c>
       <c r="C1169">
-        <v>5060</v>
+        <v>5080</v>
       </c>
       <c r="D1169" t="s">
         <v>1171</v>
@@ -22236,7 +22524,7 @@
         <v>17</v>
       </c>
       <c r="C1170">
-        <v>5070</v>
+        <v>5100</v>
       </c>
       <c r="D1170" t="s">
         <v>1172</v>
@@ -22250,7 +22538,7 @@
         <v>18</v>
       </c>
       <c r="C1171">
-        <v>5080</v>
+        <v>5100</v>
       </c>
       <c r="D1171" t="s">
         <v>1173</v>
@@ -22264,7 +22552,7 @@
         <v>19</v>
       </c>
       <c r="C1172">
-        <v>5090</v>
+        <v>5100</v>
       </c>
       <c r="D1172" t="s">
         <v>1174</v>
@@ -22278,7 +22566,7 @@
         <v>20</v>
       </c>
       <c r="C1173">
-        <v>5120</v>
+        <v>5100</v>
       </c>
       <c r="D1173" t="s">
         <v>1175</v>
@@ -22292,7 +22580,7 @@
         <v>21</v>
       </c>
       <c r="C1174">
-        <v>5150</v>
+        <v>5110</v>
       </c>
       <c r="D1174" t="s">
         <v>1176</v>
@@ -22306,7 +22594,7 @@
         <v>22</v>
       </c>
       <c r="C1175">
-        <v>5200</v>
+        <v>5140</v>
       </c>
       <c r="D1175" t="s">
         <v>1177</v>
@@ -22320,7 +22608,7 @@
         <v>23</v>
       </c>
       <c r="C1176">
-        <v>5260</v>
+        <v>5180</v>
       </c>
       <c r="D1176" t="s">
         <v>1178</v>
@@ -22334,7 +22622,7 @@
         <v>24</v>
       </c>
       <c r="C1177">
-        <v>5320</v>
+        <v>5250</v>
       </c>
       <c r="D1177" t="s">
         <v>1179</v>
@@ -22348,7 +22636,7 @@
         <v>25</v>
       </c>
       <c r="C1178">
-        <v>5400</v>
+        <v>5310</v>
       </c>
       <c r="D1178" t="s">
         <v>1180</v>
@@ -22362,7 +22650,7 @@
         <v>26</v>
       </c>
       <c r="C1179">
-        <v>5480</v>
+        <v>5410</v>
       </c>
       <c r="D1179" t="s">
         <v>1181</v>
@@ -22376,7 +22664,7 @@
         <v>27</v>
       </c>
       <c r="C1180">
-        <v>5570</v>
+        <v>5510</v>
       </c>
       <c r="D1180" t="s">
         <v>1182</v>
@@ -22390,7 +22678,7 @@
         <v>28</v>
       </c>
       <c r="C1181">
-        <v>5650</v>
+        <v>5620</v>
       </c>
       <c r="D1181" t="s">
         <v>1183</v>
@@ -22404,7 +22692,7 @@
         <v>29</v>
       </c>
       <c r="C1182">
-        <v>5740</v>
+        <v>5820</v>
       </c>
       <c r="D1182" t="s">
         <v>1184</v>
@@ -22418,7 +22706,7 @@
         <v>30</v>
       </c>
       <c r="C1183">
-        <v>5820</v>
+        <v>5950</v>
       </c>
       <c r="D1183" t="s">
         <v>1185</v>
@@ -22432,7 +22720,7 @@
         <v>31</v>
       </c>
       <c r="C1184">
-        <v>5900</v>
+        <v>6030</v>
       </c>
       <c r="D1184" t="s">
         <v>1186</v>
@@ -22446,7 +22734,7 @@
         <v>32</v>
       </c>
       <c r="C1185">
-        <v>5970</v>
+        <v>6080</v>
       </c>
       <c r="D1185" t="s">
         <v>1187</v>
@@ -22460,7 +22748,7 @@
         <v>33</v>
       </c>
       <c r="C1186">
-        <v>6030</v>
+        <v>6110</v>
       </c>
       <c r="D1186" t="s">
         <v>1188</v>
@@ -22474,7 +22762,7 @@
         <v>34</v>
       </c>
       <c r="C1187">
-        <v>6080</v>
+        <v>6100</v>
       </c>
       <c r="D1187" t="s">
         <v>1189</v>
@@ -22502,7 +22790,7 @@
         <v>36</v>
       </c>
       <c r="C1189">
-        <v>6100</v>
+        <v>6090</v>
       </c>
       <c r="D1189" t="s">
         <v>1191</v>
@@ -22516,7 +22804,7 @@
         <v>37</v>
       </c>
       <c r="C1190">
-        <v>6090</v>
+        <v>6060</v>
       </c>
       <c r="D1190" t="s">
         <v>1192</v>
@@ -22530,7 +22818,7 @@
         <v>38</v>
       </c>
       <c r="C1191">
-        <v>6060</v>
+        <v>6020</v>
       </c>
       <c r="D1191" t="s">
         <v>1193</v>
@@ -22544,7 +22832,7 @@
         <v>39</v>
       </c>
       <c r="C1192">
-        <v>6010</v>
+        <v>5990</v>
       </c>
       <c r="D1192" t="s">
         <v>1194</v>
@@ -22558,7 +22846,7 @@
         <v>40</v>
       </c>
       <c r="C1193">
-        <v>5950</v>
+        <v>5910</v>
       </c>
       <c r="D1193" t="s">
         <v>1195</v>
@@ -22572,7 +22860,7 @@
         <v>41</v>
       </c>
       <c r="C1194">
-        <v>5870</v>
+        <v>5830</v>
       </c>
       <c r="D1194" t="s">
         <v>1196</v>
@@ -22586,7 +22874,7 @@
         <v>42</v>
       </c>
       <c r="C1195">
-        <v>5800</v>
+        <v>5740</v>
       </c>
       <c r="D1195" t="s">
         <v>1197</v>
@@ -22600,7 +22888,7 @@
         <v>43</v>
       </c>
       <c r="C1196">
-        <v>5720</v>
+        <v>5650</v>
       </c>
       <c r="D1196" t="s">
         <v>1198</v>
@@ -22614,7 +22902,7 @@
         <v>44</v>
       </c>
       <c r="C1197">
-        <v>5650</v>
+        <v>5570</v>
       </c>
       <c r="D1197" t="s">
         <v>1199</v>
@@ -22628,7 +22916,7 @@
         <v>45</v>
       </c>
       <c r="C1198">
-        <v>5590</v>
+        <v>5460</v>
       </c>
       <c r="D1198" t="s">
         <v>1200</v>
@@ -22642,7 +22930,7 @@
         <v>46</v>
       </c>
       <c r="C1199">
-        <v>5540</v>
+        <v>5400</v>
       </c>
       <c r="D1199" t="s">
         <v>1201</v>
@@ -22656,7 +22944,7 @@
         <v>47</v>
       </c>
       <c r="C1200">
-        <v>5500</v>
+        <v>5350</v>
       </c>
       <c r="D1200" t="s">
         <v>1202</v>
@@ -22670,7 +22958,7 @@
         <v>48</v>
       </c>
       <c r="C1201">
-        <v>5470</v>
+        <v>5310</v>
       </c>
       <c r="D1201" t="s">
         <v>1203</v>
@@ -22684,7 +22972,7 @@
         <v>49</v>
       </c>
       <c r="C1202">
-        <v>5440</v>
+        <v>5280</v>
       </c>
       <c r="D1202" t="s">
         <v>1204</v>
@@ -22698,7 +22986,7 @@
         <v>50</v>
       </c>
       <c r="C1203">
-        <v>5420</v>
+        <v>5260</v>
       </c>
       <c r="D1203" t="s">
         <v>1205</v>
@@ -22712,7 +23000,7 @@
         <v>51</v>
       </c>
       <c r="C1204">
-        <v>5410</v>
+        <v>5240</v>
       </c>
       <c r="D1204" t="s">
         <v>1206</v>
@@ -22726,7 +23014,7 @@
         <v>52</v>
       </c>
       <c r="C1205">
-        <v>5390</v>
+        <v>5240</v>
       </c>
       <c r="D1205" t="s">
         <v>1207</v>
@@ -22740,7 +23028,7 @@
         <v>53</v>
       </c>
       <c r="C1206">
-        <v>5380</v>
+        <v>5240</v>
       </c>
       <c r="D1206" t="s">
         <v>1208</v>
@@ -22754,7 +23042,7 @@
         <v>54</v>
       </c>
       <c r="C1207">
-        <v>5380</v>
+        <v>5240</v>
       </c>
       <c r="D1207" t="s">
         <v>1209</v>
@@ -22768,7 +23056,7 @@
         <v>55</v>
       </c>
       <c r="C1208">
-        <v>5370</v>
+        <v>5240</v>
       </c>
       <c r="D1208" t="s">
         <v>1210</v>
@@ -22782,7 +23070,7 @@
         <v>56</v>
       </c>
       <c r="C1209">
-        <v>5370</v>
+        <v>5230</v>
       </c>
       <c r="D1209" t="s">
         <v>1211</v>
@@ -22796,7 +23084,7 @@
         <v>57</v>
       </c>
       <c r="C1210">
-        <v>5380</v>
+        <v>5210</v>
       </c>
       <c r="D1210" t="s">
         <v>1212</v>
@@ -22810,7 +23098,7 @@
         <v>58</v>
       </c>
       <c r="C1211">
-        <v>5390</v>
+        <v>5200</v>
       </c>
       <c r="D1211" t="s">
         <v>1213</v>
@@ -22824,7 +23112,7 @@
         <v>59</v>
       </c>
       <c r="C1212">
-        <v>5390</v>
+        <v>5200</v>
       </c>
       <c r="D1212" t="s">
         <v>1214</v>
@@ -22838,7 +23126,7 @@
         <v>60</v>
       </c>
       <c r="C1213">
-        <v>5400</v>
+        <v>5210</v>
       </c>
       <c r="D1213" t="s">
         <v>1215</v>
@@ -22852,7 +23140,7 @@
         <v>61</v>
       </c>
       <c r="C1214">
-        <v>5410</v>
+        <v>5240</v>
       </c>
       <c r="D1214" t="s">
         <v>1216</v>
@@ -22866,7 +23154,7 @@
         <v>62</v>
       </c>
       <c r="C1215">
-        <v>5410</v>
+        <v>5260</v>
       </c>
       <c r="D1215" t="s">
         <v>1217</v>
@@ -22880,7 +23168,7 @@
         <v>63</v>
       </c>
       <c r="C1216">
-        <v>5420</v>
+        <v>5280</v>
       </c>
       <c r="D1216" t="s">
         <v>1218</v>
@@ -22894,7 +23182,7 @@
         <v>64</v>
       </c>
       <c r="C1217">
-        <v>5440</v>
+        <v>5310</v>
       </c>
       <c r="D1217" t="s">
         <v>1219</v>
@@ -22908,7 +23196,7 @@
         <v>65</v>
       </c>
       <c r="C1218">
-        <v>5470</v>
+        <v>5370</v>
       </c>
       <c r="D1218" t="s">
         <v>1220</v>
@@ -22922,7 +23210,7 @@
         <v>66</v>
       </c>
       <c r="C1219">
-        <v>5510</v>
+        <v>5430</v>
       </c>
       <c r="D1219" t="s">
         <v>1221</v>
@@ -22936,7 +23224,7 @@
         <v>67</v>
       </c>
       <c r="C1220">
-        <v>5580</v>
+        <v>5500</v>
       </c>
       <c r="D1220" t="s">
         <v>1222</v>
@@ -22950,7 +23238,7 @@
         <v>68</v>
       </c>
       <c r="C1221">
-        <v>5650</v>
+        <v>5570</v>
       </c>
       <c r="D1221" t="s">
         <v>1223</v>
@@ -22964,7 +23252,7 @@
         <v>69</v>
       </c>
       <c r="C1222">
-        <v>5740</v>
+        <v>5660</v>
       </c>
       <c r="D1222" t="s">
         <v>1224</v>
@@ -22978,7 +23266,7 @@
         <v>70</v>
       </c>
       <c r="C1223">
-        <v>5840</v>
+        <v>5740</v>
       </c>
       <c r="D1223" t="s">
         <v>1225</v>
@@ -22992,7 +23280,7 @@
         <v>71</v>
       </c>
       <c r="C1224">
-        <v>5930</v>
+        <v>5810</v>
       </c>
       <c r="D1224" t="s">
         <v>1226</v>
@@ -23006,7 +23294,7 @@
         <v>72</v>
       </c>
       <c r="C1225">
-        <v>6010</v>
+        <v>5900</v>
       </c>
       <c r="D1225" t="s">
         <v>1227</v>
@@ -23020,7 +23308,7 @@
         <v>73</v>
       </c>
       <c r="C1226">
-        <v>6080</v>
+        <v>6010</v>
       </c>
       <c r="D1226" t="s">
         <v>1228</v>
@@ -23034,7 +23322,7 @@
         <v>74</v>
       </c>
       <c r="C1227">
-        <v>6160</v>
+        <v>6100</v>
       </c>
       <c r="D1227" t="s">
         <v>1229</v>
@@ -23048,7 +23336,7 @@
         <v>75</v>
       </c>
       <c r="C1228">
-        <v>6240</v>
+        <v>6190</v>
       </c>
       <c r="D1228" t="s">
         <v>1230</v>
@@ -23062,7 +23350,7 @@
         <v>76</v>
       </c>
       <c r="C1229">
-        <v>6330</v>
+        <v>6300</v>
       </c>
       <c r="D1229" t="s">
         <v>1231</v>
@@ -23076,7 +23364,7 @@
         <v>77</v>
       </c>
       <c r="C1230">
-        <v>6430</v>
+        <v>6390</v>
       </c>
       <c r="D1230" t="s">
         <v>1232</v>
@@ -23090,7 +23378,7 @@
         <v>78</v>
       </c>
       <c r="C1231">
-        <v>6540</v>
+        <v>6510</v>
       </c>
       <c r="D1231" t="s">
         <v>1233</v>
@@ -23104,7 +23392,7 @@
         <v>79</v>
       </c>
       <c r="C1232">
-        <v>6640</v>
+        <v>6610</v>
       </c>
       <c r="D1232" t="s">
         <v>1234</v>
@@ -23118,7 +23406,7 @@
         <v>80</v>
       </c>
       <c r="C1233">
-        <v>6720</v>
+        <v>6690</v>
       </c>
       <c r="D1233" t="s">
         <v>1235</v>
@@ -23132,7 +23420,7 @@
         <v>81</v>
       </c>
       <c r="C1234">
-        <v>6810</v>
+        <v>6780</v>
       </c>
       <c r="D1234" t="s">
         <v>1236</v>
@@ -23146,7 +23434,7 @@
         <v>82</v>
       </c>
       <c r="C1235">
-        <v>6910</v>
+        <v>6860</v>
       </c>
       <c r="D1235" t="s">
         <v>1237</v>
@@ -23160,7 +23448,7 @@
         <v>83</v>
       </c>
       <c r="C1236">
-        <v>6980</v>
+        <v>6910</v>
       </c>
       <c r="D1236" t="s">
         <v>1238</v>
@@ -23174,7 +23462,7 @@
         <v>84</v>
       </c>
       <c r="C1237">
-        <v>7030</v>
+        <v>6970</v>
       </c>
       <c r="D1237" t="s">
         <v>1239</v>
@@ -23188,7 +23476,7 @@
         <v>85</v>
       </c>
       <c r="C1238">
-        <v>7050</v>
+        <v>7010</v>
       </c>
       <c r="D1238" t="s">
         <v>1240</v>
@@ -23202,7 +23490,7 @@
         <v>86</v>
       </c>
       <c r="C1239">
-        <v>7050</v>
+        <v>6980</v>
       </c>
       <c r="D1239" t="s">
         <v>1241</v>
@@ -23216,7 +23504,7 @@
         <v>87</v>
       </c>
       <c r="C1240">
-        <v>7030</v>
+        <v>6920</v>
       </c>
       <c r="D1240" t="s">
         <v>1242</v>
@@ -23230,7 +23518,7 @@
         <v>88</v>
       </c>
       <c r="C1241">
-        <v>6980</v>
+        <v>6810</v>
       </c>
       <c r="D1241" t="s">
         <v>1243</v>
@@ -23244,7 +23532,7 @@
         <v>89</v>
       </c>
       <c r="C1242">
-        <v>6860</v>
+        <v>6650</v>
       </c>
       <c r="D1242" t="s">
         <v>1244</v>
@@ -23258,7 +23546,7 @@
         <v>90</v>
       </c>
       <c r="C1243">
-        <v>6730</v>
+        <v>6500</v>
       </c>
       <c r="D1243" t="s">
         <v>1245</v>
@@ -23272,7 +23560,7 @@
         <v>91</v>
       </c>
       <c r="C1244">
-        <v>6550</v>
+        <v>6350</v>
       </c>
       <c r="D1244" t="s">
         <v>1246</v>
@@ -23286,7 +23574,7 @@
         <v>92</v>
       </c>
       <c r="C1245">
-        <v>6360</v>
+        <v>6190</v>
       </c>
       <c r="D1245" t="s">
         <v>1247</v>
@@ -23300,7 +23588,7 @@
         <v>93</v>
       </c>
       <c r="C1246">
-        <v>6180</v>
+        <v>6020</v>
       </c>
       <c r="D1246" t="s">
         <v>1248</v>
@@ -23314,7 +23602,7 @@
         <v>94</v>
       </c>
       <c r="C1247">
-        <v>6020</v>
+        <v>5860</v>
       </c>
       <c r="D1247" t="s">
         <v>1249</v>
@@ -23328,7 +23616,7 @@
         <v>95</v>
       </c>
       <c r="C1248">
-        <v>5880</v>
+        <v>5750</v>
       </c>
       <c r="D1248" t="s">
         <v>1250</v>
@@ -23342,7 +23630,7 @@
         <v>96</v>
       </c>
       <c r="C1249">
-        <v>5740</v>
+        <v>5640</v>
       </c>
       <c r="D1249" t="s">
         <v>1251</v>
@@ -23356,7 +23644,7 @@
         <v>1</v>
       </c>
       <c r="C1250">
-        <v>5480</v>
+        <v>5430</v>
       </c>
       <c r="D1250" t="s">
         <v>1252</v>
@@ -23370,7 +23658,7 @@
         <v>2</v>
       </c>
       <c r="C1251">
-        <v>5420</v>
+        <v>5330</v>
       </c>
       <c r="D1251" t="s">
         <v>1253</v>
@@ -23384,7 +23672,7 @@
         <v>3</v>
       </c>
       <c r="C1252">
-        <v>5350</v>
+        <v>5260</v>
       </c>
       <c r="D1252" t="s">
         <v>1254</v>
@@ -23398,7 +23686,7 @@
         <v>4</v>
       </c>
       <c r="C1253">
-        <v>5300</v>
+        <v>5200</v>
       </c>
       <c r="D1253" t="s">
         <v>1255</v>
@@ -23412,7 +23700,7 @@
         <v>5</v>
       </c>
       <c r="C1254">
-        <v>5240</v>
+        <v>5150</v>
       </c>
       <c r="D1254" t="s">
         <v>1256</v>
@@ -23426,7 +23714,7 @@
         <v>6</v>
       </c>
       <c r="C1255">
-        <v>5210</v>
+        <v>5100</v>
       </c>
       <c r="D1255" t="s">
         <v>1257</v>
@@ -23440,7 +23728,7 @@
         <v>7</v>
       </c>
       <c r="C1256">
-        <v>5180</v>
+        <v>5090</v>
       </c>
       <c r="D1256" t="s">
         <v>1258</v>
@@ -23454,7 +23742,7 @@
         <v>8</v>
       </c>
       <c r="C1257">
-        <v>5130</v>
+        <v>5060</v>
       </c>
       <c r="D1257" t="s">
         <v>1259</v>
@@ -23468,7 +23756,7 @@
         <v>9</v>
       </c>
       <c r="C1258">
-        <v>5090</v>
+        <v>5050</v>
       </c>
       <c r="D1258" t="s">
         <v>1260</v>
@@ -23482,7 +23770,7 @@
         <v>10</v>
       </c>
       <c r="C1259">
-        <v>5050</v>
+        <v>5040</v>
       </c>
       <c r="D1259" t="s">
         <v>1261</v>
@@ -23496,7 +23784,7 @@
         <v>11</v>
       </c>
       <c r="C1260">
-        <v>5030</v>
+        <v>5040</v>
       </c>
       <c r="D1260" t="s">
         <v>1262</v>
@@ -23510,7 +23798,7 @@
         <v>12</v>
       </c>
       <c r="C1261">
-        <v>5020</v>
+        <v>5040</v>
       </c>
       <c r="D1261" t="s">
         <v>1263</v>
@@ -23524,7 +23812,7 @@
         <v>13</v>
       </c>
       <c r="C1262">
-        <v>5020</v>
+        <v>5030</v>
       </c>
       <c r="D1262" t="s">
         <v>1264</v>
@@ -23538,7 +23826,7 @@
         <v>14</v>
       </c>
       <c r="C1263">
-        <v>5030</v>
+        <v>5020</v>
       </c>
       <c r="D1263" t="s">
         <v>1265</v>
@@ -23552,7 +23840,7 @@
         <v>15</v>
       </c>
       <c r="C1264">
-        <v>5040</v>
+        <v>5020</v>
       </c>
       <c r="D1264" t="s">
         <v>1266</v>
@@ -23566,7 +23854,7 @@
         <v>16</v>
       </c>
       <c r="C1265">
-        <v>5050</v>
+        <v>5030</v>
       </c>
       <c r="D1265" t="s">
         <v>1267</v>
@@ -23580,7 +23868,7 @@
         <v>17</v>
       </c>
       <c r="C1266">
-        <v>5050</v>
+        <v>5060</v>
       </c>
       <c r="D1266" t="s">
         <v>1268</v>
@@ -23594,7 +23882,7 @@
         <v>18</v>
       </c>
       <c r="C1267">
-        <v>5060</v>
+        <v>5070</v>
       </c>
       <c r="D1267" t="s">
         <v>1269</v>
@@ -23622,7 +23910,7 @@
         <v>20</v>
       </c>
       <c r="C1269">
-        <v>5090</v>
+        <v>5100</v>
       </c>
       <c r="D1269" t="s">
         <v>1271</v>
@@ -23636,7 +23924,7 @@
         <v>21</v>
       </c>
       <c r="C1270">
-        <v>5120</v>
+        <v>5110</v>
       </c>
       <c r="D1270" t="s">
         <v>1272</v>
@@ -23650,7 +23938,7 @@
         <v>22</v>
       </c>
       <c r="C1271">
-        <v>5170</v>
+        <v>5120</v>
       </c>
       <c r="D1271" t="s">
         <v>1273</v>
@@ -23664,7 +23952,7 @@
         <v>23</v>
       </c>
       <c r="C1272">
-        <v>5240</v>
+        <v>5150</v>
       </c>
       <c r="D1272" t="s">
         <v>1274</v>
@@ -23678,7 +23966,7 @@
         <v>24</v>
       </c>
       <c r="C1273">
-        <v>5330</v>
+        <v>5210</v>
       </c>
       <c r="D1273" t="s">
         <v>1275</v>
@@ -23692,7 +23980,7 @@
         <v>25</v>
       </c>
       <c r="C1274">
-        <v>5430</v>
+        <v>5290</v>
       </c>
       <c r="D1274" t="s">
         <v>1276</v>
@@ -23706,7 +23994,7 @@
         <v>26</v>
       </c>
       <c r="C1275">
-        <v>5540</v>
+        <v>5360</v>
       </c>
       <c r="D1275" t="s">
         <v>1277</v>
@@ -23720,7 +24008,7 @@
         <v>27</v>
       </c>
       <c r="C1276">
-        <v>5650</v>
+        <v>5470</v>
       </c>
       <c r="D1276" t="s">
         <v>1278</v>
@@ -23734,7 +24022,7 @@
         <v>28</v>
       </c>
       <c r="C1277">
-        <v>5750</v>
+        <v>5590</v>
       </c>
       <c r="D1277" t="s">
         <v>1279</v>
@@ -23748,7 +24036,7 @@
         <v>29</v>
       </c>
       <c r="C1278">
-        <v>5840</v>
+        <v>5730</v>
       </c>
       <c r="D1278" t="s">
         <v>1280</v>
@@ -23762,7 +24050,7 @@
         <v>30</v>
       </c>
       <c r="C1279">
-        <v>5920</v>
+        <v>5840</v>
       </c>
       <c r="D1279" t="s">
         <v>1281</v>
@@ -23776,7 +24064,7 @@
         <v>31</v>
       </c>
       <c r="C1280">
-        <v>5970</v>
+        <v>5900</v>
       </c>
       <c r="D1280" t="s">
         <v>1282</v>
@@ -23790,7 +24078,7 @@
         <v>32</v>
       </c>
       <c r="C1281">
-        <v>6010</v>
+        <v>5920</v>
       </c>
       <c r="D1281" t="s">
         <v>1283</v>
@@ -23804,7 +24092,7 @@
         <v>33</v>
       </c>
       <c r="C1282">
-        <v>6010</v>
+        <v>5920</v>
       </c>
       <c r="D1282" t="s">
         <v>1284</v>
@@ -23818,7 +24106,7 @@
         <v>34</v>
       </c>
       <c r="C1283">
-        <v>5990</v>
+        <v>5900</v>
       </c>
       <c r="D1283" t="s">
         <v>1285</v>
@@ -23832,7 +24120,7 @@
         <v>35</v>
       </c>
       <c r="C1284">
-        <v>5950</v>
+        <v>5840</v>
       </c>
       <c r="D1284" t="s">
         <v>1286</v>
@@ -23846,7 +24134,7 @@
         <v>36</v>
       </c>
       <c r="C1285">
-        <v>5880</v>
+        <v>5730</v>
       </c>
       <c r="D1285" t="s">
         <v>1287</v>
@@ -23860,7 +24148,7 @@
         <v>37</v>
       </c>
       <c r="C1286">
-        <v>5790</v>
+        <v>5610</v>
       </c>
       <c r="D1286" t="s">
         <v>1288</v>
@@ -23874,7 +24162,7 @@
         <v>38</v>
       </c>
       <c r="C1287">
-        <v>5690</v>
+        <v>5500</v>
       </c>
       <c r="D1287" t="s">
         <v>1289</v>
@@ -23888,7 +24176,7 @@
         <v>39</v>
       </c>
       <c r="C1288">
-        <v>5570</v>
+        <v>5370</v>
       </c>
       <c r="D1288" t="s">
         <v>1290</v>
@@ -23902,7 +24190,7 @@
         <v>40</v>
       </c>
       <c r="C1289">
-        <v>5450</v>
+        <v>5230</v>
       </c>
       <c r="D1289" t="s">
         <v>1291</v>
@@ -23916,7 +24204,7 @@
         <v>41</v>
       </c>
       <c r="C1290">
-        <v>5330</v>
+        <v>5120</v>
       </c>
       <c r="D1290" t="s">
         <v>1292</v>
@@ -23930,7 +24218,7 @@
         <v>42</v>
       </c>
       <c r="C1291">
-        <v>5220</v>
+        <v>5000</v>
       </c>
       <c r="D1291" t="s">
         <v>1293</v>
@@ -23944,7 +24232,7 @@
         <v>43</v>
       </c>
       <c r="C1292">
-        <v>5110</v>
+        <v>4890</v>
       </c>
       <c r="D1292" t="s">
         <v>1294</v>
@@ -23958,7 +24246,7 @@
         <v>44</v>
       </c>
       <c r="C1293">
-        <v>5020</v>
+        <v>4790</v>
       </c>
       <c r="D1293" t="s">
         <v>1295</v>
@@ -23972,7 +24260,7 @@
         <v>45</v>
       </c>
       <c r="C1294">
-        <v>4940</v>
+        <v>4670</v>
       </c>
       <c r="D1294" t="s">
         <v>1296</v>
@@ -23986,7 +24274,7 @@
         <v>46</v>
       </c>
       <c r="C1295">
-        <v>4880</v>
+        <v>4600</v>
       </c>
       <c r="D1295" t="s">
         <v>1297</v>
@@ -24000,7 +24288,7 @@
         <v>47</v>
       </c>
       <c r="C1296">
-        <v>4830</v>
+        <v>4550</v>
       </c>
       <c r="D1296" t="s">
         <v>1298</v>
@@ -24014,7 +24302,7 @@
         <v>48</v>
       </c>
       <c r="C1297">
-        <v>4790</v>
+        <v>4500</v>
       </c>
       <c r="D1297" t="s">
         <v>1299</v>
@@ -24028,7 +24316,7 @@
         <v>49</v>
       </c>
       <c r="C1298">
-        <v>4770</v>
+        <v>4440</v>
       </c>
       <c r="D1298" t="s">
         <v>1300</v>
@@ -24042,7 +24330,7 @@
         <v>50</v>
       </c>
       <c r="C1299">
-        <v>4750</v>
+        <v>4410</v>
       </c>
       <c r="D1299" t="s">
         <v>1301</v>
@@ -24056,7 +24344,7 @@
         <v>51</v>
       </c>
       <c r="C1300">
-        <v>4740</v>
+        <v>4390</v>
       </c>
       <c r="D1300" t="s">
         <v>1302</v>
@@ -24070,7 +24358,7 @@
         <v>52</v>
       </c>
       <c r="C1301">
-        <v>4740</v>
+        <v>4380</v>
       </c>
       <c r="D1301" t="s">
         <v>1303</v>
@@ -24084,7 +24372,7 @@
         <v>53</v>
       </c>
       <c r="C1302">
-        <v>4740</v>
+        <v>4390</v>
       </c>
       <c r="D1302" t="s">
         <v>1304</v>
@@ -24098,7 +24386,7 @@
         <v>54</v>
       </c>
       <c r="C1303">
-        <v>4750</v>
+        <v>4390</v>
       </c>
       <c r="D1303" t="s">
         <v>1305</v>
@@ -24112,7 +24400,7 @@
         <v>55</v>
       </c>
       <c r="C1304">
-        <v>4760</v>
+        <v>4400</v>
       </c>
       <c r="D1304" t="s">
         <v>1306</v>
@@ -24126,7 +24414,7 @@
         <v>56</v>
       </c>
       <c r="C1305">
-        <v>4780</v>
+        <v>4400</v>
       </c>
       <c r="D1305" t="s">
         <v>1307</v>
@@ -24140,7 +24428,7 @@
         <v>57</v>
       </c>
       <c r="C1306">
-        <v>4810</v>
+        <v>4420</v>
       </c>
       <c r="D1306" t="s">
         <v>1308</v>
@@ -24154,7 +24442,7 @@
         <v>58</v>
       </c>
       <c r="C1307">
-        <v>4840</v>
+        <v>4430</v>
       </c>
       <c r="D1307" t="s">
         <v>1309</v>
@@ -24168,7 +24456,7 @@
         <v>59</v>
       </c>
       <c r="C1308">
-        <v>4870</v>
+        <v>4440</v>
       </c>
       <c r="D1308" t="s">
         <v>1310</v>
@@ -24182,7 +24470,7 @@
         <v>60</v>
       </c>
       <c r="C1309">
-        <v>4900</v>
+        <v>4450</v>
       </c>
       <c r="D1309" t="s">
         <v>1311</v>
@@ -24196,7 +24484,7 @@
         <v>61</v>
       </c>
       <c r="C1310">
-        <v>4940</v>
+        <v>4490</v>
       </c>
       <c r="D1310" t="s">
         <v>1312</v>
@@ -24210,7 +24498,7 @@
         <v>62</v>
       </c>
       <c r="C1311">
-        <v>4980</v>
+        <v>4520</v>
       </c>
       <c r="D1311" t="s">
         <v>1313</v>
@@ -24224,7 +24512,7 @@
         <v>63</v>
       </c>
       <c r="C1312">
-        <v>5020</v>
+        <v>4550</v>
       </c>
       <c r="D1312" t="s">
         <v>1314</v>
@@ -24238,7 +24526,7 @@
         <v>64</v>
       </c>
       <c r="C1313">
-        <v>5080</v>
+        <v>4600</v>
       </c>
       <c r="D1313" t="s">
         <v>1315</v>
@@ -24252,7 +24540,7 @@
         <v>65</v>
       </c>
       <c r="C1314">
-        <v>5150</v>
+        <v>4660</v>
       </c>
       <c r="D1314" t="s">
         <v>1316</v>
@@ -24266,7 +24554,7 @@
         <v>66</v>
       </c>
       <c r="C1315">
-        <v>5240</v>
+        <v>4730</v>
       </c>
       <c r="D1315" t="s">
         <v>1317</v>
@@ -24280,7 +24568,7 @@
         <v>67</v>
       </c>
       <c r="C1316">
-        <v>5340</v>
+        <v>4830</v>
       </c>
       <c r="D1316" t="s">
         <v>1318</v>
@@ -24294,7 +24582,7 @@
         <v>68</v>
       </c>
       <c r="C1317">
-        <v>5440</v>
+        <v>4920</v>
       </c>
       <c r="D1317" t="s">
         <v>1319</v>
@@ -24308,7 +24596,7 @@
         <v>69</v>
       </c>
       <c r="C1318">
-        <v>5550</v>
+        <v>5020</v>
       </c>
       <c r="D1318" t="s">
         <v>1320</v>
@@ -24322,7 +24610,7 @@
         <v>70</v>
       </c>
       <c r="C1319">
-        <v>5660</v>
+        <v>5110</v>
       </c>
       <c r="D1319" t="s">
         <v>1321</v>
@@ -24336,7 +24624,7 @@
         <v>71</v>
       </c>
       <c r="C1320">
-        <v>5770</v>
+        <v>5220</v>
       </c>
       <c r="D1320" t="s">
         <v>1322</v>
@@ -24350,7 +24638,7 @@
         <v>72</v>
       </c>
       <c r="C1321">
-        <v>5880</v>
+        <v>5350</v>
       </c>
       <c r="D1321" t="s">
         <v>1323</v>
@@ -24364,7 +24652,7 @@
         <v>73</v>
       </c>
       <c r="C1322">
-        <v>5970</v>
+        <v>5500</v>
       </c>
       <c r="D1322" t="s">
         <v>1324</v>
@@ -24378,7 +24666,7 @@
         <v>74</v>
       </c>
       <c r="C1323">
-        <v>6060</v>
+        <v>5650</v>
       </c>
       <c r="D1323" t="s">
         <v>1325</v>
@@ -24392,7 +24680,7 @@
         <v>75</v>
       </c>
       <c r="C1324">
-        <v>6160</v>
+        <v>5800</v>
       </c>
       <c r="D1324" t="s">
         <v>1326</v>
@@ -24406,7 +24694,7 @@
         <v>76</v>
       </c>
       <c r="C1325">
-        <v>6270</v>
+        <v>5940</v>
       </c>
       <c r="D1325" t="s">
         <v>1327</v>
@@ -24420,7 +24708,7 @@
         <v>77</v>
       </c>
       <c r="C1326">
-        <v>6390</v>
+        <v>6100</v>
       </c>
       <c r="D1326" t="s">
         <v>1328</v>
@@ -24434,7 +24722,7 @@
         <v>78</v>
       </c>
       <c r="C1327">
-        <v>6500</v>
+        <v>6250</v>
       </c>
       <c r="D1327" t="s">
         <v>1329</v>
@@ -24448,7 +24736,7 @@
         <v>79</v>
       </c>
       <c r="C1328">
-        <v>6600</v>
+        <v>6390</v>
       </c>
       <c r="D1328" t="s">
         <v>1330</v>
@@ -24462,7 +24750,7 @@
         <v>80</v>
       </c>
       <c r="C1329">
-        <v>6670</v>
+        <v>6530</v>
       </c>
       <c r="D1329" t="s">
         <v>1331</v>
@@ -24476,7 +24764,7 @@
         <v>81</v>
       </c>
       <c r="C1330">
-        <v>6740</v>
+        <v>6630</v>
       </c>
       <c r="D1330" t="s">
         <v>1332</v>
@@ -24490,7 +24778,7 @@
         <v>82</v>
       </c>
       <c r="C1331">
-        <v>6820</v>
+        <v>6720</v>
       </c>
       <c r="D1331" t="s">
         <v>1333</v>
@@ -24504,7 +24792,7 @@
         <v>83</v>
       </c>
       <c r="C1332">
-        <v>6890</v>
+        <v>6790</v>
       </c>
       <c r="D1332" t="s">
         <v>1334</v>
@@ -24518,7 +24806,7 @@
         <v>84</v>
       </c>
       <c r="C1333">
-        <v>6980</v>
+        <v>6880</v>
       </c>
       <c r="D1333" t="s">
         <v>1335</v>
@@ -24532,7 +24820,7 @@
         <v>85</v>
       </c>
       <c r="C1334">
-        <v>7020</v>
+        <v>6940</v>
       </c>
       <c r="D1334" t="s">
         <v>1336</v>
@@ -24546,7 +24834,7 @@
         <v>86</v>
       </c>
       <c r="C1335">
-        <v>7010</v>
+        <v>6940</v>
       </c>
       <c r="D1335" t="s">
         <v>1337</v>
@@ -24560,7 +24848,7 @@
         <v>87</v>
       </c>
       <c r="C1336">
-        <v>6990</v>
+        <v>6930</v>
       </c>
       <c r="D1336" t="s">
         <v>1338</v>
@@ -24574,7 +24862,7 @@
         <v>88</v>
       </c>
       <c r="C1337">
-        <v>6890</v>
+        <v>6870</v>
       </c>
       <c r="D1337" t="s">
         <v>1339</v>
@@ -24588,7 +24876,7 @@
         <v>89</v>
       </c>
       <c r="C1338">
-        <v>6750</v>
+        <v>6720</v>
       </c>
       <c r="D1338" t="s">
         <v>1340</v>
@@ -24602,7 +24890,7 @@
         <v>90</v>
       </c>
       <c r="C1339">
-        <v>6620</v>
+        <v>6520</v>
       </c>
       <c r="D1339" t="s">
         <v>1341</v>
@@ -24616,7 +24904,7 @@
         <v>91</v>
       </c>
       <c r="C1340">
-        <v>6460</v>
+        <v>6350</v>
       </c>
       <c r="D1340" t="s">
         <v>1342</v>
@@ -24630,7 +24918,7 @@
         <v>92</v>
       </c>
       <c r="C1341">
-        <v>6280</v>
+        <v>6170</v>
       </c>
       <c r="D1341" t="s">
         <v>1343</v>
@@ -24644,7 +24932,7 @@
         <v>93</v>
       </c>
       <c r="C1342">
-        <v>6120</v>
+        <v>6030</v>
       </c>
       <c r="D1342" t="s">
         <v>1344</v>
@@ -24658,7 +24946,7 @@
         <v>94</v>
       </c>
       <c r="C1343">
-        <v>5970</v>
+        <v>5890</v>
       </c>
       <c r="D1343" t="s">
         <v>1345</v>
@@ -24672,7 +24960,7 @@
         <v>95</v>
       </c>
       <c r="C1344">
-        <v>5850</v>
+        <v>5780</v>
       </c>
       <c r="D1344" t="s">
         <v>1346</v>
@@ -24686,7 +24974,7 @@
         <v>96</v>
       </c>
       <c r="C1345">
-        <v>5720</v>
+        <v>5660</v>
       </c>
       <c r="D1345" t="s">
         <v>1347</v>
@@ -24700,7 +24988,7 @@
         <v>1</v>
       </c>
       <c r="C1346">
-        <v>5470</v>
+        <v>5460</v>
       </c>
       <c r="D1346" t="s">
         <v>1348</v>
@@ -24728,7 +25016,7 @@
         <v>3</v>
       </c>
       <c r="C1348">
-        <v>5340</v>
+        <v>5360</v>
       </c>
       <c r="D1348" t="s">
         <v>1350</v>
@@ -24742,7 +25030,7 @@
         <v>4</v>
       </c>
       <c r="C1349">
-        <v>5280</v>
+        <v>5290</v>
       </c>
       <c r="D1349" t="s">
         <v>1351</v>
@@ -24756,7 +25044,7 @@
         <v>5</v>
       </c>
       <c r="C1350">
-        <v>5230</v>
+        <v>5240</v>
       </c>
       <c r="D1350" t="s">
         <v>1352</v>
@@ -24784,7 +25072,7 @@
         <v>7</v>
       </c>
       <c r="C1352">
-        <v>5160</v>
+        <v>5140</v>
       </c>
       <c r="D1352" t="s">
         <v>1354</v>
@@ -24798,7 +25086,7 @@
         <v>8</v>
       </c>
       <c r="C1353">
-        <v>5120</v>
+        <v>5100</v>
       </c>
       <c r="D1353" t="s">
         <v>1355</v>
@@ -24812,7 +25100,7 @@
         <v>9</v>
       </c>
       <c r="C1354">
-        <v>5080</v>
+        <v>5060</v>
       </c>
       <c r="D1354" t="s">
         <v>1356</v>
@@ -24826,7 +25114,7 @@
         <v>10</v>
       </c>
       <c r="C1355">
-        <v>5050</v>
+        <v>5030</v>
       </c>
       <c r="D1355" t="s">
         <v>1357</v>
@@ -24840,7 +25128,7 @@
         <v>11</v>
       </c>
       <c r="C1356">
-        <v>5040</v>
+        <v>5010</v>
       </c>
       <c r="D1356" t="s">
         <v>1358</v>
@@ -24854,7 +25142,7 @@
         <v>12</v>
       </c>
       <c r="C1357">
-        <v>5030</v>
+        <v>5010</v>
       </c>
       <c r="D1357" t="s">
         <v>1359</v>
@@ -24868,7 +25156,7 @@
         <v>13</v>
       </c>
       <c r="C1358">
-        <v>5030</v>
+        <v>5000</v>
       </c>
       <c r="D1358" t="s">
         <v>1360</v>
@@ -24882,7 +25170,7 @@
         <v>14</v>
       </c>
       <c r="C1359">
-        <v>5030</v>
+        <v>5020</v>
       </c>
       <c r="D1359" t="s">
         <v>1361</v>
@@ -24896,7 +25184,7 @@
         <v>15</v>
       </c>
       <c r="C1360">
-        <v>5040</v>
+        <v>5030</v>
       </c>
       <c r="D1360" t="s">
         <v>1362</v>
@@ -24910,7 +25198,7 @@
         <v>16</v>
       </c>
       <c r="C1361">
-        <v>5040</v>
+        <v>5030</v>
       </c>
       <c r="D1361" t="s">
         <v>1363</v>
@@ -24924,7 +25212,7 @@
         <v>17</v>
       </c>
       <c r="C1362">
-        <v>5050</v>
+        <v>5040</v>
       </c>
       <c r="D1362" t="s">
         <v>1364</v>
@@ -25008,7 +25296,7 @@
         <v>23</v>
       </c>
       <c r="C1368">
-        <v>5240</v>
+        <v>5250</v>
       </c>
       <c r="D1368" t="s">
         <v>1370</v>
@@ -25022,7 +25310,7 @@
         <v>24</v>
       </c>
       <c r="C1369">
-        <v>5310</v>
+        <v>5330</v>
       </c>
       <c r="D1369" t="s">
         <v>1371</v>
@@ -25036,7 +25324,7 @@
         <v>25</v>
       </c>
       <c r="C1370">
-        <v>5390</v>
+        <v>5410</v>
       </c>
       <c r="D1370" t="s">
         <v>1372</v>
@@ -25050,7 +25338,7 @@
         <v>26</v>
       </c>
       <c r="C1371">
-        <v>5480</v>
+        <v>5500</v>
       </c>
       <c r="D1371" t="s">
         <v>1373</v>
@@ -25064,7 +25352,7 @@
         <v>27</v>
       </c>
       <c r="C1372">
-        <v>5560</v>
+        <v>5590</v>
       </c>
       <c r="D1372" t="s">
         <v>1374</v>
@@ -25078,7 +25366,7 @@
         <v>28</v>
       </c>
       <c r="C1373">
-        <v>5640</v>
+        <v>5660</v>
       </c>
       <c r="D1373" t="s">
         <v>1375</v>
@@ -25092,7 +25380,7 @@
         <v>29</v>
       </c>
       <c r="C1374">
-        <v>5710</v>
+        <v>5720</v>
       </c>
       <c r="D1374" t="s">
         <v>1376</v>
@@ -25106,7 +25394,7 @@
         <v>30</v>
       </c>
       <c r="C1375">
-        <v>5770</v>
+        <v>5760</v>
       </c>
       <c r="D1375" t="s">
         <v>1377</v>
@@ -25120,7 +25408,7 @@
         <v>31</v>
       </c>
       <c r="C1376">
-        <v>5810</v>
+        <v>5780</v>
       </c>
       <c r="D1376" t="s">
         <v>1378</v>
@@ -25134,7 +25422,7 @@
         <v>32</v>
       </c>
       <c r="C1377">
-        <v>5830</v>
+        <v>5800</v>
       </c>
       <c r="D1377" t="s">
         <v>1379</v>
@@ -25148,7 +25436,7 @@
         <v>33</v>
       </c>
       <c r="C1378">
-        <v>5830</v>
+        <v>5750</v>
       </c>
       <c r="D1378" t="s">
         <v>1380</v>
@@ -25162,7 +25450,7 @@
         <v>34</v>
       </c>
       <c r="C1379">
-        <v>5810</v>
+        <v>5700</v>
       </c>
       <c r="D1379" t="s">
         <v>1381</v>
@@ -25176,7 +25464,7 @@
         <v>35</v>
       </c>
       <c r="C1380">
-        <v>5760</v>
+        <v>5630</v>
       </c>
       <c r="D1380" t="s">
         <v>1382</v>
@@ -25190,7 +25478,7 @@
         <v>36</v>
       </c>
       <c r="C1381">
-        <v>5700</v>
+        <v>5550</v>
       </c>
       <c r="D1381" t="s">
         <v>1383</v>
@@ -25204,7 +25492,7 @@
         <v>37</v>
       </c>
       <c r="C1382">
-        <v>5610</v>
+        <v>5460</v>
       </c>
       <c r="D1382" t="s">
         <v>1384</v>
@@ -25218,7 +25506,7 @@
         <v>38</v>
       </c>
       <c r="C1383">
-        <v>5510</v>
+        <v>5360</v>
       </c>
       <c r="D1383" t="s">
         <v>1385</v>
@@ -25232,7 +25520,7 @@
         <v>39</v>
       </c>
       <c r="C1384">
-        <v>5390</v>
+        <v>5260</v>
       </c>
       <c r="D1384" t="s">
         <v>1386</v>
@@ -25246,7 +25534,7 @@
         <v>40</v>
       </c>
       <c r="C1385">
-        <v>5270</v>
+        <v>5170</v>
       </c>
       <c r="D1385" t="s">
         <v>1387</v>
@@ -25260,7 +25548,7 @@
         <v>41</v>
       </c>
       <c r="C1386">
-        <v>5150</v>
+        <v>5080</v>
       </c>
       <c r="D1386" t="s">
         <v>1388</v>
@@ -25274,7 +25562,7 @@
         <v>42</v>
       </c>
       <c r="C1387">
-        <v>5030</v>
+        <v>4990</v>
       </c>
       <c r="D1387" t="s">
         <v>1389</v>
@@ -25288,7 +25576,7 @@
         <v>43</v>
       </c>
       <c r="C1388">
-        <v>4930</v>
+        <v>4910</v>
       </c>
       <c r="D1388" t="s">
         <v>1390</v>
@@ -25302,7 +25590,7 @@
         <v>44</v>
       </c>
       <c r="C1389">
-        <v>4840</v>
+        <v>4850</v>
       </c>
       <c r="D1389" t="s">
         <v>1391</v>
@@ -25316,7 +25604,7 @@
         <v>45</v>
       </c>
       <c r="C1390">
-        <v>4770</v>
+        <v>4780</v>
       </c>
       <c r="D1390" t="s">
         <v>1392</v>
@@ -25330,7 +25618,7 @@
         <v>46</v>
       </c>
       <c r="C1391">
-        <v>4720</v>
+        <v>4730</v>
       </c>
       <c r="D1391" t="s">
         <v>1393</v>
@@ -25358,7 +25646,7 @@
         <v>48</v>
       </c>
       <c r="C1393">
-        <v>4650</v>
+        <v>4630</v>
       </c>
       <c r="D1393" t="s">
         <v>1395</v>
@@ -25372,7 +25660,7 @@
         <v>49</v>
       </c>
       <c r="C1394">
-        <v>4630</v>
+        <v>4590</v>
       </c>
       <c r="D1394" t="s">
         <v>1396</v>
@@ -25386,7 +25674,7 @@
         <v>50</v>
       </c>
       <c r="C1395">
-        <v>4610</v>
+        <v>4550</v>
       </c>
       <c r="D1395" t="s">
         <v>1397</v>
@@ -25400,7 +25688,7 @@
         <v>51</v>
       </c>
       <c r="C1396">
-        <v>4590</v>
+        <v>4510</v>
       </c>
       <c r="D1396" t="s">
         <v>1398</v>
@@ -25414,7 +25702,7 @@
         <v>52</v>
       </c>
       <c r="C1397">
-        <v>4580</v>
+        <v>4480</v>
       </c>
       <c r="D1397" t="s">
         <v>1399</v>
@@ -25428,7 +25716,7 @@
         <v>53</v>
       </c>
       <c r="C1398">
-        <v>4560</v>
+        <v>4450</v>
       </c>
       <c r="D1398" t="s">
         <v>1400</v>
@@ -25442,7 +25730,7 @@
         <v>54</v>
       </c>
       <c r="C1399">
-        <v>4540</v>
+        <v>4430</v>
       </c>
       <c r="D1399" t="s">
         <v>1401</v>
@@ -25456,7 +25744,7 @@
         <v>55</v>
       </c>
       <c r="C1400">
-        <v>4540</v>
+        <v>4420</v>
       </c>
       <c r="D1400" t="s">
         <v>1402</v>
@@ -25470,7 +25758,7 @@
         <v>56</v>
       </c>
       <c r="C1401">
-        <v>4540</v>
+        <v>4420</v>
       </c>
       <c r="D1401" t="s">
         <v>1403</v>
@@ -25484,7 +25772,7 @@
         <v>57</v>
       </c>
       <c r="C1402">
-        <v>4550</v>
+        <v>4430</v>
       </c>
       <c r="D1402" t="s">
         <v>1404</v>
@@ -25498,7 +25786,7 @@
         <v>58</v>
       </c>
       <c r="C1403">
-        <v>4570</v>
+        <v>4450</v>
       </c>
       <c r="D1403" t="s">
         <v>1405</v>
@@ -25512,7 +25800,7 @@
         <v>59</v>
       </c>
       <c r="C1404">
-        <v>4600</v>
+        <v>4480</v>
       </c>
       <c r="D1404" t="s">
         <v>1406</v>
@@ -25526,7 +25814,7 @@
         <v>60</v>
       </c>
       <c r="C1405">
-        <v>4650</v>
+        <v>4510</v>
       </c>
       <c r="D1405" t="s">
         <v>1407</v>
@@ -25540,7 +25828,7 @@
         <v>61</v>
       </c>
       <c r="C1406">
-        <v>4700</v>
+        <v>4550</v>
       </c>
       <c r="D1406" t="s">
         <v>1408</v>
@@ -25554,7 +25842,7 @@
         <v>62</v>
       </c>
       <c r="C1407">
-        <v>4770</v>
+        <v>4590</v>
       </c>
       <c r="D1407" t="s">
         <v>1409</v>
@@ -25568,7 +25856,7 @@
         <v>63</v>
       </c>
       <c r="C1408">
-        <v>4840</v>
+        <v>4640</v>
       </c>
       <c r="D1408" t="s">
         <v>1410</v>
@@ -25582,7 +25870,7 @@
         <v>64</v>
       </c>
       <c r="C1409">
-        <v>4910</v>
+        <v>4700</v>
       </c>
       <c r="D1409" t="s">
         <v>1411</v>
@@ -25596,7 +25884,7 @@
         <v>65</v>
       </c>
       <c r="C1410">
-        <v>5000</v>
+        <v>4770</v>
       </c>
       <c r="D1410" t="s">
         <v>1412</v>
@@ -25610,7 +25898,7 @@
         <v>66</v>
       </c>
       <c r="C1411">
-        <v>5100</v>
+        <v>4850</v>
       </c>
       <c r="D1411" t="s">
         <v>1413</v>
@@ -25624,7 +25912,7 @@
         <v>67</v>
       </c>
       <c r="C1412">
-        <v>5210</v>
+        <v>4940</v>
       </c>
       <c r="D1412" t="s">
         <v>1414</v>
@@ -25638,7 +25926,7 @@
         <v>68</v>
       </c>
       <c r="C1413">
-        <v>5320</v>
+        <v>5050</v>
       </c>
       <c r="D1413" t="s">
         <v>1415</v>
@@ -25652,7 +25940,7 @@
         <v>69</v>
       </c>
       <c r="C1414">
-        <v>5440</v>
+        <v>5160</v>
       </c>
       <c r="D1414" t="s">
         <v>1416</v>
@@ -25666,7 +25954,7 @@
         <v>70</v>
       </c>
       <c r="C1415">
-        <v>5550</v>
+        <v>5270</v>
       </c>
       <c r="D1415" t="s">
         <v>1417</v>
@@ -25680,7 +25968,7 @@
         <v>71</v>
       </c>
       <c r="C1416">
-        <v>5650</v>
+        <v>5380</v>
       </c>
       <c r="D1416" t="s">
         <v>1418</v>
@@ -25694,7 +25982,7 @@
         <v>72</v>
       </c>
       <c r="C1417">
-        <v>5750</v>
+        <v>5490</v>
       </c>
       <c r="D1417" t="s">
         <v>1419</v>
@@ -25708,7 +25996,7 @@
         <v>73</v>
       </c>
       <c r="C1418">
-        <v>5840</v>
+        <v>5610</v>
       </c>
       <c r="D1418" t="s">
         <v>1420</v>
@@ -25722,7 +26010,7 @@
         <v>74</v>
       </c>
       <c r="C1419">
-        <v>5930</v>
+        <v>5720</v>
       </c>
       <c r="D1419" t="s">
         <v>1421</v>
@@ -25736,7 +26024,7 @@
         <v>75</v>
       </c>
       <c r="C1420">
-        <v>6040</v>
+        <v>5850</v>
       </c>
       <c r="D1420" t="s">
         <v>1422</v>
@@ -25750,7 +26038,7 @@
         <v>76</v>
       </c>
       <c r="C1421">
-        <v>6150</v>
+        <v>5980</v>
       </c>
       <c r="D1421" t="s">
         <v>1423</v>
@@ -25764,7 +26052,7 @@
         <v>77</v>
       </c>
       <c r="C1422">
-        <v>6280</v>
+        <v>6120</v>
       </c>
       <c r="D1422" t="s">
         <v>1424</v>
@@ -25778,7 +26066,7 @@
         <v>78</v>
       </c>
       <c r="C1423">
-        <v>6400</v>
+        <v>6260</v>
       </c>
       <c r="D1423" t="s">
         <v>1425</v>
@@ -25792,7 +26080,7 @@
         <v>79</v>
       </c>
       <c r="C1424">
-        <v>6500</v>
+        <v>6390</v>
       </c>
       <c r="D1424" t="s">
         <v>1426</v>
@@ -25806,7 +26094,7 @@
         <v>80</v>
       </c>
       <c r="C1425">
-        <v>6570</v>
+        <v>6490</v>
       </c>
       <c r="D1425" t="s">
         <v>1427</v>
@@ -25820,7 +26108,7 @@
         <v>81</v>
       </c>
       <c r="C1426">
-        <v>6650</v>
+        <v>6600</v>
       </c>
       <c r="D1426" t="s">
         <v>1428</v>
@@ -25834,7 +26122,7 @@
         <v>82</v>
       </c>
       <c r="C1427">
-        <v>6720</v>
+        <v>6660</v>
       </c>
       <c r="D1427" t="s">
         <v>1429</v>
@@ -25848,7 +26136,7 @@
         <v>83</v>
       </c>
       <c r="C1428">
-        <v>6790</v>
+        <v>6720</v>
       </c>
       <c r="D1428" t="s">
         <v>1430</v>
@@ -25862,7 +26150,7 @@
         <v>84</v>
       </c>
       <c r="C1429">
-        <v>6880</v>
+        <v>6750</v>
       </c>
       <c r="D1429" t="s">
         <v>1431</v>
@@ -25876,7 +26164,7 @@
         <v>85</v>
       </c>
       <c r="C1430">
-        <v>6920</v>
+        <v>6750</v>
       </c>
       <c r="D1430" t="s">
         <v>1432</v>
@@ -25890,7 +26178,7 @@
         <v>86</v>
       </c>
       <c r="C1431">
-        <v>6910</v>
+        <v>6750</v>
       </c>
       <c r="D1431" t="s">
         <v>1433</v>
@@ -25904,7 +26192,7 @@
         <v>87</v>
       </c>
       <c r="C1432">
-        <v>6890</v>
+        <v>6720</v>
       </c>
       <c r="D1432" t="s">
         <v>1434</v>
@@ -25918,7 +26206,7 @@
         <v>88</v>
       </c>
       <c r="C1433">
-        <v>6790</v>
+        <v>6650</v>
       </c>
       <c r="D1433" t="s">
         <v>1435</v>
@@ -25932,7 +26220,7 @@
         <v>89</v>
       </c>
       <c r="C1434">
-        <v>6650</v>
+        <v>6520</v>
       </c>
       <c r="D1434" t="s">
         <v>1436</v>
@@ -25946,7 +26234,7 @@
         <v>90</v>
       </c>
       <c r="C1435">
-        <v>6520</v>
+        <v>6430</v>
       </c>
       <c r="D1435" t="s">
         <v>1437</v>
@@ -25960,7 +26248,7 @@
         <v>91</v>
       </c>
       <c r="C1436">
-        <v>6360</v>
+        <v>6270</v>
       </c>
       <c r="D1436" t="s">
         <v>1438</v>
@@ -25974,7 +26262,7 @@
         <v>92</v>
       </c>
       <c r="C1437">
-        <v>6190</v>
+        <v>6140</v>
       </c>
       <c r="D1437" t="s">
         <v>1439</v>
@@ -25988,7 +26276,7 @@
         <v>93</v>
       </c>
       <c r="C1438">
-        <v>6030</v>
+        <v>5980</v>
       </c>
       <c r="D1438" t="s">
         <v>1440</v>
@@ -26002,7 +26290,7 @@
         <v>94</v>
       </c>
       <c r="C1439">
-        <v>5880</v>
+        <v>5820</v>
       </c>
       <c r="D1439" t="s">
         <v>1441</v>
@@ -26016,7 +26304,7 @@
         <v>95</v>
       </c>
       <c r="C1440">
-        <v>5750</v>
+        <v>5730</v>
       </c>
       <c r="D1440" t="s">
         <v>1442</v>
@@ -31410,6 +31698,1350 @@
       </c>
       <c r="D1825" t="s">
         <v>1827</v>
+      </c>
+    </row>
+    <row r="1826" spans="1:4">
+      <c r="A1826" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1826">
+        <v>1</v>
+      </c>
+      <c r="C1826">
+        <v>5620</v>
+      </c>
+      <c r="D1826" t="s">
+        <v>1828</v>
+      </c>
+    </row>
+    <row r="1827" spans="1:4">
+      <c r="A1827" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1827">
+        <v>2</v>
+      </c>
+      <c r="C1827">
+        <v>5580</v>
+      </c>
+      <c r="D1827" t="s">
+        <v>1829</v>
+      </c>
+    </row>
+    <row r="1828" spans="1:4">
+      <c r="A1828" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1828">
+        <v>3</v>
+      </c>
+      <c r="C1828">
+        <v>5520</v>
+      </c>
+      <c r="D1828" t="s">
+        <v>1830</v>
+      </c>
+    </row>
+    <row r="1829" spans="1:4">
+      <c r="A1829" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1829">
+        <v>4</v>
+      </c>
+      <c r="C1829">
+        <v>5440</v>
+      </c>
+      <c r="D1829" t="s">
+        <v>1831</v>
+      </c>
+    </row>
+    <row r="1830" spans="1:4">
+      <c r="A1830" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1830">
+        <v>5</v>
+      </c>
+      <c r="C1830">
+        <v>5370</v>
+      </c>
+      <c r="D1830" t="s">
+        <v>1832</v>
+      </c>
+    </row>
+    <row r="1831" spans="1:4">
+      <c r="A1831" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1831">
+        <v>6</v>
+      </c>
+      <c r="C1831">
+        <v>5320</v>
+      </c>
+      <c r="D1831" t="s">
+        <v>1833</v>
+      </c>
+    </row>
+    <row r="1832" spans="1:4">
+      <c r="A1832" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1832">
+        <v>7</v>
+      </c>
+      <c r="C1832">
+        <v>5280</v>
+      </c>
+      <c r="D1832" t="s">
+        <v>1834</v>
+      </c>
+    </row>
+    <row r="1833" spans="1:4">
+      <c r="A1833" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1833">
+        <v>8</v>
+      </c>
+      <c r="C1833">
+        <v>5240</v>
+      </c>
+      <c r="D1833" t="s">
+        <v>1835</v>
+      </c>
+    </row>
+    <row r="1834" spans="1:4">
+      <c r="A1834" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1834">
+        <v>9</v>
+      </c>
+      <c r="C1834">
+        <v>5210</v>
+      </c>
+      <c r="D1834" t="s">
+        <v>1836</v>
+      </c>
+    </row>
+    <row r="1835" spans="1:4">
+      <c r="A1835" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1835">
+        <v>10</v>
+      </c>
+      <c r="C1835">
+        <v>5190</v>
+      </c>
+      <c r="D1835" t="s">
+        <v>1837</v>
+      </c>
+    </row>
+    <row r="1836" spans="1:4">
+      <c r="A1836" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1836">
+        <v>11</v>
+      </c>
+      <c r="C1836">
+        <v>5170</v>
+      </c>
+      <c r="D1836" t="s">
+        <v>1838</v>
+      </c>
+    </row>
+    <row r="1837" spans="1:4">
+      <c r="A1837" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1837">
+        <v>12</v>
+      </c>
+      <c r="C1837">
+        <v>5150</v>
+      </c>
+      <c r="D1837" t="s">
+        <v>1839</v>
+      </c>
+    </row>
+    <row r="1838" spans="1:4">
+      <c r="A1838" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1838">
+        <v>13</v>
+      </c>
+      <c r="C1838">
+        <v>5150</v>
+      </c>
+      <c r="D1838" t="s">
+        <v>1840</v>
+      </c>
+    </row>
+    <row r="1839" spans="1:4">
+      <c r="A1839" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1839">
+        <v>14</v>
+      </c>
+      <c r="C1839">
+        <v>5150</v>
+      </c>
+      <c r="D1839" t="s">
+        <v>1841</v>
+      </c>
+    </row>
+    <row r="1840" spans="1:4">
+      <c r="A1840" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1840">
+        <v>15</v>
+      </c>
+      <c r="C1840">
+        <v>5150</v>
+      </c>
+      <c r="D1840" t="s">
+        <v>1842</v>
+      </c>
+    </row>
+    <row r="1841" spans="1:4">
+      <c r="A1841" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1841">
+        <v>16</v>
+      </c>
+      <c r="C1841">
+        <v>5160</v>
+      </c>
+      <c r="D1841" t="s">
+        <v>1843</v>
+      </c>
+    </row>
+    <row r="1842" spans="1:4">
+      <c r="A1842" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1842">
+        <v>17</v>
+      </c>
+      <c r="C1842">
+        <v>5160</v>
+      </c>
+      <c r="D1842" t="s">
+        <v>1844</v>
+      </c>
+    </row>
+    <row r="1843" spans="1:4">
+      <c r="A1843" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1843">
+        <v>18</v>
+      </c>
+      <c r="C1843">
+        <v>5160</v>
+      </c>
+      <c r="D1843" t="s">
+        <v>1845</v>
+      </c>
+    </row>
+    <row r="1844" spans="1:4">
+      <c r="A1844" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1844">
+        <v>19</v>
+      </c>
+      <c r="C1844">
+        <v>5170</v>
+      </c>
+      <c r="D1844" t="s">
+        <v>1846</v>
+      </c>
+    </row>
+    <row r="1845" spans="1:4">
+      <c r="A1845" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1845">
+        <v>20</v>
+      </c>
+      <c r="C1845">
+        <v>5180</v>
+      </c>
+      <c r="D1845" t="s">
+        <v>1847</v>
+      </c>
+    </row>
+    <row r="1846" spans="1:4">
+      <c r="A1846" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1846">
+        <v>21</v>
+      </c>
+      <c r="C1846">
+        <v>5200</v>
+      </c>
+      <c r="D1846" t="s">
+        <v>1848</v>
+      </c>
+    </row>
+    <row r="1847" spans="1:4">
+      <c r="A1847" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1847">
+        <v>22</v>
+      </c>
+      <c r="C1847">
+        <v>5230</v>
+      </c>
+      <c r="D1847" t="s">
+        <v>1849</v>
+      </c>
+    </row>
+    <row r="1848" spans="1:4">
+      <c r="A1848" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1848">
+        <v>23</v>
+      </c>
+      <c r="C1848">
+        <v>5290</v>
+      </c>
+      <c r="D1848" t="s">
+        <v>1850</v>
+      </c>
+    </row>
+    <row r="1849" spans="1:4">
+      <c r="A1849" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1849">
+        <v>24</v>
+      </c>
+      <c r="C1849">
+        <v>5360</v>
+      </c>
+      <c r="D1849" t="s">
+        <v>1851</v>
+      </c>
+    </row>
+    <row r="1850" spans="1:4">
+      <c r="A1850" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1850">
+        <v>25</v>
+      </c>
+      <c r="C1850">
+        <v>5460</v>
+      </c>
+      <c r="D1850" t="s">
+        <v>1852</v>
+      </c>
+    </row>
+    <row r="1851" spans="1:4">
+      <c r="A1851" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1851">
+        <v>26</v>
+      </c>
+      <c r="C1851">
+        <v>5570</v>
+      </c>
+      <c r="D1851" t="s">
+        <v>1853</v>
+      </c>
+    </row>
+    <row r="1852" spans="1:4">
+      <c r="A1852" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1852">
+        <v>27</v>
+      </c>
+      <c r="C1852">
+        <v>5690</v>
+      </c>
+      <c r="D1852" t="s">
+        <v>1854</v>
+      </c>
+    </row>
+    <row r="1853" spans="1:4">
+      <c r="A1853" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1853">
+        <v>28</v>
+      </c>
+      <c r="C1853">
+        <v>5810</v>
+      </c>
+      <c r="D1853" t="s">
+        <v>1855</v>
+      </c>
+    </row>
+    <row r="1854" spans="1:4">
+      <c r="A1854" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1854">
+        <v>29</v>
+      </c>
+      <c r="C1854">
+        <v>5930</v>
+      </c>
+      <c r="D1854" t="s">
+        <v>1856</v>
+      </c>
+    </row>
+    <row r="1855" spans="1:4">
+      <c r="A1855" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1855">
+        <v>30</v>
+      </c>
+      <c r="C1855">
+        <v>6040</v>
+      </c>
+      <c r="D1855" t="s">
+        <v>1857</v>
+      </c>
+    </row>
+    <row r="1856" spans="1:4">
+      <c r="A1856" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1856">
+        <v>31</v>
+      </c>
+      <c r="C1856">
+        <v>6120</v>
+      </c>
+      <c r="D1856" t="s">
+        <v>1858</v>
+      </c>
+    </row>
+    <row r="1857" spans="1:4">
+      <c r="A1857" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1857">
+        <v>32</v>
+      </c>
+      <c r="C1857">
+        <v>6170</v>
+      </c>
+      <c r="D1857" t="s">
+        <v>1859</v>
+      </c>
+    </row>
+    <row r="1858" spans="1:4">
+      <c r="A1858" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1858">
+        <v>33</v>
+      </c>
+      <c r="C1858">
+        <v>6200</v>
+      </c>
+      <c r="D1858" t="s">
+        <v>1860</v>
+      </c>
+    </row>
+    <row r="1859" spans="1:4">
+      <c r="A1859" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1859">
+        <v>34</v>
+      </c>
+      <c r="C1859">
+        <v>6190</v>
+      </c>
+      <c r="D1859" t="s">
+        <v>1861</v>
+      </c>
+    </row>
+    <row r="1860" spans="1:4">
+      <c r="A1860" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1860">
+        <v>35</v>
+      </c>
+      <c r="C1860">
+        <v>6150</v>
+      </c>
+      <c r="D1860" t="s">
+        <v>1862</v>
+      </c>
+    </row>
+    <row r="1861" spans="1:4">
+      <c r="A1861" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1861">
+        <v>36</v>
+      </c>
+      <c r="C1861">
+        <v>6090</v>
+      </c>
+      <c r="D1861" t="s">
+        <v>1863</v>
+      </c>
+    </row>
+    <row r="1862" spans="1:4">
+      <c r="A1862" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1862">
+        <v>37</v>
+      </c>
+      <c r="C1862">
+        <v>6010</v>
+      </c>
+      <c r="D1862" t="s">
+        <v>1864</v>
+      </c>
+    </row>
+    <row r="1863" spans="1:4">
+      <c r="A1863" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1863">
+        <v>38</v>
+      </c>
+      <c r="C1863">
+        <v>5910</v>
+      </c>
+      <c r="D1863" t="s">
+        <v>1865</v>
+      </c>
+    </row>
+    <row r="1864" spans="1:4">
+      <c r="A1864" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1864">
+        <v>39</v>
+      </c>
+      <c r="C1864">
+        <v>5810</v>
+      </c>
+      <c r="D1864" t="s">
+        <v>1866</v>
+      </c>
+    </row>
+    <row r="1865" spans="1:4">
+      <c r="A1865" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1865">
+        <v>40</v>
+      </c>
+      <c r="C1865">
+        <v>5700</v>
+      </c>
+      <c r="D1865" t="s">
+        <v>1867</v>
+      </c>
+    </row>
+    <row r="1866" spans="1:4">
+      <c r="A1866" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1866">
+        <v>41</v>
+      </c>
+      <c r="C1866">
+        <v>5590</v>
+      </c>
+      <c r="D1866" t="s">
+        <v>1868</v>
+      </c>
+    </row>
+    <row r="1867" spans="1:4">
+      <c r="A1867" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1867">
+        <v>42</v>
+      </c>
+      <c r="C1867">
+        <v>5500</v>
+      </c>
+      <c r="D1867" t="s">
+        <v>1869</v>
+      </c>
+    </row>
+    <row r="1868" spans="1:4">
+      <c r="A1868" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1868">
+        <v>43</v>
+      </c>
+      <c r="C1868">
+        <v>5410</v>
+      </c>
+      <c r="D1868" t="s">
+        <v>1870</v>
+      </c>
+    </row>
+    <row r="1869" spans="1:4">
+      <c r="A1869" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1869">
+        <v>44</v>
+      </c>
+      <c r="C1869">
+        <v>5330</v>
+      </c>
+      <c r="D1869" t="s">
+        <v>1871</v>
+      </c>
+    </row>
+    <row r="1870" spans="1:4">
+      <c r="A1870" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1870">
+        <v>45</v>
+      </c>
+      <c r="C1870">
+        <v>5250</v>
+      </c>
+      <c r="D1870" t="s">
+        <v>1872</v>
+      </c>
+    </row>
+    <row r="1871" spans="1:4">
+      <c r="A1871" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1871">
+        <v>46</v>
+      </c>
+      <c r="C1871">
+        <v>5190</v>
+      </c>
+      <c r="D1871" t="s">
+        <v>1873</v>
+      </c>
+    </row>
+    <row r="1872" spans="1:4">
+      <c r="A1872" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1872">
+        <v>47</v>
+      </c>
+      <c r="C1872">
+        <v>5140</v>
+      </c>
+      <c r="D1872" t="s">
+        <v>1874</v>
+      </c>
+    </row>
+    <row r="1873" spans="1:4">
+      <c r="A1873" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1873">
+        <v>48</v>
+      </c>
+      <c r="C1873">
+        <v>5090</v>
+      </c>
+      <c r="D1873" t="s">
+        <v>1875</v>
+      </c>
+    </row>
+    <row r="1874" spans="1:4">
+      <c r="A1874" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1874">
+        <v>49</v>
+      </c>
+      <c r="C1874">
+        <v>5050</v>
+      </c>
+      <c r="D1874" t="s">
+        <v>1876</v>
+      </c>
+    </row>
+    <row r="1875" spans="1:4">
+      <c r="A1875" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1875">
+        <v>50</v>
+      </c>
+      <c r="C1875">
+        <v>5010</v>
+      </c>
+      <c r="D1875" t="s">
+        <v>1877</v>
+      </c>
+    </row>
+    <row r="1876" spans="1:4">
+      <c r="A1876" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1876">
+        <v>51</v>
+      </c>
+      <c r="C1876">
+        <v>4990</v>
+      </c>
+      <c r="D1876" t="s">
+        <v>1878</v>
+      </c>
+    </row>
+    <row r="1877" spans="1:4">
+      <c r="A1877" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1877">
+        <v>52</v>
+      </c>
+      <c r="C1877">
+        <v>4970</v>
+      </c>
+      <c r="D1877" t="s">
+        <v>1879</v>
+      </c>
+    </row>
+    <row r="1878" spans="1:4">
+      <c r="A1878" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1878">
+        <v>53</v>
+      </c>
+      <c r="C1878">
+        <v>4960</v>
+      </c>
+      <c r="D1878" t="s">
+        <v>1880</v>
+      </c>
+    </row>
+    <row r="1879" spans="1:4">
+      <c r="A1879" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1879">
+        <v>54</v>
+      </c>
+      <c r="C1879">
+        <v>4960</v>
+      </c>
+      <c r="D1879" t="s">
+        <v>1881</v>
+      </c>
+    </row>
+    <row r="1880" spans="1:4">
+      <c r="A1880" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1880">
+        <v>55</v>
+      </c>
+      <c r="C1880">
+        <v>4960</v>
+      </c>
+      <c r="D1880" t="s">
+        <v>1882</v>
+      </c>
+    </row>
+    <row r="1881" spans="1:4">
+      <c r="A1881" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1881">
+        <v>56</v>
+      </c>
+      <c r="C1881">
+        <v>4970</v>
+      </c>
+      <c r="D1881" t="s">
+        <v>1883</v>
+      </c>
+    </row>
+    <row r="1882" spans="1:4">
+      <c r="A1882" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1882">
+        <v>57</v>
+      </c>
+      <c r="C1882">
+        <v>4990</v>
+      </c>
+      <c r="D1882" t="s">
+        <v>1884</v>
+      </c>
+    </row>
+    <row r="1883" spans="1:4">
+      <c r="A1883" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1883">
+        <v>58</v>
+      </c>
+      <c r="C1883">
+        <v>5000</v>
+      </c>
+      <c r="D1883" t="s">
+        <v>1885</v>
+      </c>
+    </row>
+    <row r="1884" spans="1:4">
+      <c r="A1884" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1884">
+        <v>59</v>
+      </c>
+      <c r="C1884">
+        <v>5020</v>
+      </c>
+      <c r="D1884" t="s">
+        <v>1886</v>
+      </c>
+    </row>
+    <row r="1885" spans="1:4">
+      <c r="A1885" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1885">
+        <v>60</v>
+      </c>
+      <c r="C1885">
+        <v>5040</v>
+      </c>
+      <c r="D1885" t="s">
+        <v>1887</v>
+      </c>
+    </row>
+    <row r="1886" spans="1:4">
+      <c r="A1886" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1886">
+        <v>61</v>
+      </c>
+      <c r="C1886">
+        <v>5070</v>
+      </c>
+      <c r="D1886" t="s">
+        <v>1888</v>
+      </c>
+    </row>
+    <row r="1887" spans="1:4">
+      <c r="A1887" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1887">
+        <v>62</v>
+      </c>
+      <c r="C1887">
+        <v>5110</v>
+      </c>
+      <c r="D1887" t="s">
+        <v>1889</v>
+      </c>
+    </row>
+    <row r="1888" spans="1:4">
+      <c r="A1888" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1888">
+        <v>63</v>
+      </c>
+      <c r="C1888">
+        <v>5160</v>
+      </c>
+      <c r="D1888" t="s">
+        <v>1890</v>
+      </c>
+    </row>
+    <row r="1889" spans="1:4">
+      <c r="A1889" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1889">
+        <v>64</v>
+      </c>
+      <c r="C1889">
+        <v>5220</v>
+      </c>
+      <c r="D1889" t="s">
+        <v>1891</v>
+      </c>
+    </row>
+    <row r="1890" spans="1:4">
+      <c r="A1890" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1890">
+        <v>65</v>
+      </c>
+      <c r="C1890">
+        <v>5300</v>
+      </c>
+      <c r="D1890" t="s">
+        <v>1892</v>
+      </c>
+    </row>
+    <row r="1891" spans="1:4">
+      <c r="A1891" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1891">
+        <v>66</v>
+      </c>
+      <c r="C1891">
+        <v>5380</v>
+      </c>
+      <c r="D1891" t="s">
+        <v>1893</v>
+      </c>
+    </row>
+    <row r="1892" spans="1:4">
+      <c r="A1892" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1892">
+        <v>67</v>
+      </c>
+      <c r="C1892">
+        <v>5470</v>
+      </c>
+      <c r="D1892" t="s">
+        <v>1894</v>
+      </c>
+    </row>
+    <row r="1893" spans="1:4">
+      <c r="A1893" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1893">
+        <v>68</v>
+      </c>
+      <c r="C1893">
+        <v>5560</v>
+      </c>
+      <c r="D1893" t="s">
+        <v>1895</v>
+      </c>
+    </row>
+    <row r="1894" spans="1:4">
+      <c r="A1894" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1894">
+        <v>69</v>
+      </c>
+      <c r="C1894">
+        <v>5640</v>
+      </c>
+      <c r="D1894" t="s">
+        <v>1896</v>
+      </c>
+    </row>
+    <row r="1895" spans="1:4">
+      <c r="A1895" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1895">
+        <v>70</v>
+      </c>
+      <c r="C1895">
+        <v>5720</v>
+      </c>
+      <c r="D1895" t="s">
+        <v>1897</v>
+      </c>
+    </row>
+    <row r="1896" spans="1:4">
+      <c r="A1896" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1896">
+        <v>71</v>
+      </c>
+      <c r="C1896">
+        <v>5800</v>
+      </c>
+      <c r="D1896" t="s">
+        <v>1898</v>
+      </c>
+    </row>
+    <row r="1897" spans="1:4">
+      <c r="A1897" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1897">
+        <v>72</v>
+      </c>
+      <c r="C1897">
+        <v>5880</v>
+      </c>
+      <c r="D1897" t="s">
+        <v>1899</v>
+      </c>
+    </row>
+    <row r="1898" spans="1:4">
+      <c r="A1898" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1898">
+        <v>73</v>
+      </c>
+      <c r="C1898">
+        <v>5970</v>
+      </c>
+      <c r="D1898" t="s">
+        <v>1900</v>
+      </c>
+    </row>
+    <row r="1899" spans="1:4">
+      <c r="A1899" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1899">
+        <v>74</v>
+      </c>
+      <c r="C1899">
+        <v>6070</v>
+      </c>
+      <c r="D1899" t="s">
+        <v>1901</v>
+      </c>
+    </row>
+    <row r="1900" spans="1:4">
+      <c r="A1900" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1900">
+        <v>75</v>
+      </c>
+      <c r="C1900">
+        <v>6180</v>
+      </c>
+      <c r="D1900" t="s">
+        <v>1902</v>
+      </c>
+    </row>
+    <row r="1901" spans="1:4">
+      <c r="A1901" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1901">
+        <v>76</v>
+      </c>
+      <c r="C1901">
+        <v>6300</v>
+      </c>
+      <c r="D1901" t="s">
+        <v>1903</v>
+      </c>
+    </row>
+    <row r="1902" spans="1:4">
+      <c r="A1902" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1902">
+        <v>77</v>
+      </c>
+      <c r="C1902">
+        <v>6430</v>
+      </c>
+      <c r="D1902" t="s">
+        <v>1904</v>
+      </c>
+    </row>
+    <row r="1903" spans="1:4">
+      <c r="A1903" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1903">
+        <v>78</v>
+      </c>
+      <c r="C1903">
+        <v>6560</v>
+      </c>
+      <c r="D1903" t="s">
+        <v>1905</v>
+      </c>
+    </row>
+    <row r="1904" spans="1:4">
+      <c r="A1904" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1904">
+        <v>79</v>
+      </c>
+      <c r="C1904">
+        <v>6660</v>
+      </c>
+      <c r="D1904" t="s">
+        <v>1906</v>
+      </c>
+    </row>
+    <row r="1905" spans="1:4">
+      <c r="A1905" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1905">
+        <v>80</v>
+      </c>
+      <c r="C1905">
+        <v>6750</v>
+      </c>
+      <c r="D1905" t="s">
+        <v>1907</v>
+      </c>
+    </row>
+    <row r="1906" spans="1:4">
+      <c r="A1906" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1906">
+        <v>81</v>
+      </c>
+      <c r="C1906">
+        <v>6850</v>
+      </c>
+      <c r="D1906" t="s">
+        <v>1908</v>
+      </c>
+    </row>
+    <row r="1907" spans="1:4">
+      <c r="A1907" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1907">
+        <v>82</v>
+      </c>
+      <c r="C1907">
+        <v>6950</v>
+      </c>
+      <c r="D1907" t="s">
+        <v>1909</v>
+      </c>
+    </row>
+    <row r="1908" spans="1:4">
+      <c r="A1908" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1908">
+        <v>83</v>
+      </c>
+      <c r="C1908">
+        <v>7030</v>
+      </c>
+      <c r="D1908" t="s">
+        <v>1910</v>
+      </c>
+    </row>
+    <row r="1909" spans="1:4">
+      <c r="A1909" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1909">
+        <v>84</v>
+      </c>
+      <c r="C1909">
+        <v>7090</v>
+      </c>
+      <c r="D1909" t="s">
+        <v>1911</v>
+      </c>
+    </row>
+    <row r="1910" spans="1:4">
+      <c r="A1910" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1910">
+        <v>85</v>
+      </c>
+      <c r="C1910">
+        <v>7080</v>
+      </c>
+      <c r="D1910" t="s">
+        <v>1912</v>
+      </c>
+    </row>
+    <row r="1911" spans="1:4">
+      <c r="A1911" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1911">
+        <v>86</v>
+      </c>
+      <c r="C1911">
+        <v>7020</v>
+      </c>
+      <c r="D1911" t="s">
+        <v>1913</v>
+      </c>
+    </row>
+    <row r="1912" spans="1:4">
+      <c r="A1912" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1912">
+        <v>87</v>
+      </c>
+      <c r="C1912">
+        <v>7000</v>
+      </c>
+      <c r="D1912" t="s">
+        <v>1914</v>
+      </c>
+    </row>
+    <row r="1913" spans="1:4">
+      <c r="A1913" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1913">
+        <v>88</v>
+      </c>
+      <c r="C1913">
+        <v>6960</v>
+      </c>
+      <c r="D1913" t="s">
+        <v>1915</v>
+      </c>
+    </row>
+    <row r="1914" spans="1:4">
+      <c r="A1914" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1914">
+        <v>89</v>
+      </c>
+      <c r="C1914">
+        <v>6890</v>
+      </c>
+      <c r="D1914" t="s">
+        <v>1916</v>
+      </c>
+    </row>
+    <row r="1915" spans="1:4">
+      <c r="A1915" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1915">
+        <v>90</v>
+      </c>
+      <c r="C1915">
+        <v>6840</v>
+      </c>
+      <c r="D1915" t="s">
+        <v>1917</v>
+      </c>
+    </row>
+    <row r="1916" spans="1:4">
+      <c r="A1916" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1916">
+        <v>91</v>
+      </c>
+      <c r="C1916">
+        <v>6690</v>
+      </c>
+      <c r="D1916" t="s">
+        <v>1918</v>
+      </c>
+    </row>
+    <row r="1917" spans="1:4">
+      <c r="A1917" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1917">
+        <v>92</v>
+      </c>
+      <c r="C1917">
+        <v>6500</v>
+      </c>
+      <c r="D1917" t="s">
+        <v>1919</v>
+      </c>
+    </row>
+    <row r="1918" spans="1:4">
+      <c r="A1918" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1918">
+        <v>93</v>
+      </c>
+      <c r="C1918">
+        <v>6280</v>
+      </c>
+      <c r="D1918" t="s">
+        <v>1920</v>
+      </c>
+    </row>
+    <row r="1919" spans="1:4">
+      <c r="A1919" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1919">
+        <v>94</v>
+      </c>
+      <c r="C1919">
+        <v>6090</v>
+      </c>
+      <c r="D1919" t="s">
+        <v>1921</v>
+      </c>
+    </row>
+    <row r="1920" spans="1:4">
+      <c r="A1920" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1920">
+        <v>95</v>
+      </c>
+      <c r="C1920">
+        <v>6010</v>
+      </c>
+      <c r="D1920" t="s">
+        <v>1922</v>
+      </c>
+    </row>
+    <row r="1921" spans="1:4">
+      <c r="A1921" s="2">
+        <v>46162</v>
+      </c>
+      <c r="B1921">
+        <v>96</v>
+      </c>
+      <c r="C1921">
+        <v>5900</v>
+      </c>
+      <c r="D1921" t="s">
+        <v>1923</v>
       </c>
     </row>
   </sheetData>

</xml_diff>